<commit_message>
US English throughout the repository prose, parameter tables and workbook notes
license, summarize, realized, artifact, data center, modeled, judgment etc., to match
the paper. Parameter name market_based_intensity_realised -> _realized. Left verbatim:
the engine code, launcher and scheduled prompts that ran the campaign (the measurement
prompt is quoted in paper Appendix B.3), the corpus, and the prompt_class value
'summarise'. Expected tables regenerated (text only); numbers unchanged.

Checks: Corpus 644/644; bootstrap and ratio envelopes 0.0000; 1,971/1,971 paper cells;
3,954 formulas, 0 undeclared constants.

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/workbooks/OpenAIModelCalculations_v1.0.0.xlsx
+++ b/data/workbooks/OpenAIModelCalculations_v1.0.0.xlsx
@@ -81,7 +81,7 @@
     <t xml:space="preserve">Table 3 / Section 4.7</t>
   </si>
   <si>
-    <t xml:space="preserve">Market-based intensity gCO2e/Wh (Stargate credited at Oracle FY25 corporate 46 gCO2e/kWh; Google credited at CY2025 realised market-based Scope 2 — Section 4.8)</t>
+    <t xml:space="preserve">Market-based intensity gCO2e/Wh (Stargate credited at Oracle FY25 corporate 46 gCO2e/kWh; Google credited at CY2025 realized market-based Scope 2 — Section 4.8)</t>
   </si>
   <si>
     <t xml:space="preserve">Table 5 / Section 4.8 — computed in GridIntensity!F20</t>
@@ -150,7 +150,7 @@
     <t xml:space="preserve">Corpus provenance: InferenceCarbon_corpus_frozen_20260822.zip, SHA-256 01c57eb5bf41476fee8e06a8b677a72c172c849741cc65a9b554cf7397d84cc6. Copyright (c) 2026 InferenceCarbon Ltd.</t>
   </si>
   <si>
-    <t xml:space="preserve">GridIntensity — Tables 3, 4, 5 and 10 (Sections 4.5 – 4.8, 5.4). Typed values are inputs; every other number is a formula. Google is credited at its GHG Protocol 2015 market-based Scope 2 realised intensity (Google 2026 Environmental Report, CY2025).</t>
+    <t xml:space="preserve">GridIntensity — Tables 3, 4, 5 and 10 (Sections 4.5 – 4.8, 5.4). Typed values are inputs; every other number is a formula. Google is credited at its GHG Protocol 2015 market-based Scope 2 realized intensity (Google 2026 Environmental Report, CY2025).</t>
   </si>
   <si>
     <t xml:space="preserve">Google inputs (2026 Environmental Report, Environmental metrics data tables, pp. 89, 92)</t>
@@ -171,7 +171,7 @@
     <t xml:space="preserve">Total electricity consumption, CY2025 (MWh)</t>
   </si>
   <si>
-    <t xml:space="preserve">Google 2026 Environmental Report, p. 92 (data centres 42,415,800 MWh = 97.3%)</t>
+    <t xml:space="preserve">Google 2026 Environmental Report, p. 92 (data centers 42,415,800 MWh = 97.3%)</t>
   </si>
   <si>
     <t xml:space="preserve">Scope 2 market-based, CY2024 (tCO2e)</t>
@@ -183,25 +183,25 @@
     <t xml:space="preserve">Google 2026 Environmental Report, p. 92</t>
   </si>
   <si>
-    <t xml:space="preserve">Hourly CFE, data centres, CY2025 (%)</t>
+    <t xml:space="preserve">Hourly CFE, data centers, CY2025 (%)</t>
   </si>
   <si>
     <t xml:space="preserve">Google 2026 Environmental Report, p. 93 — reported alongside, not instead of, market-based Scope 2; not used in Table 4</t>
   </si>
   <si>
-    <t xml:space="preserve">Google realised market-based intensity, CY2025 (gCO2e/kWh)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">tCO2e × 1e6 / (MWh × 1e3) — Section 3.7 realised-intensity rule, as applied to Microsoft [32] and Oracle [16]</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Google realised location-based intensity, CY2025 (gCO2e/kWh)</t>
+    <t xml:space="preserve">Google realized market-based intensity, CY2025 (gCO2e/kWh)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">tCO2e × 1e6 / (MWh × 1e3) — Section 3.7 realized-intensity rule, as applied to Microsoft [32] and Oracle [16]</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Google realized location-based intensity, CY2025 (gCO2e/kWh)</t>
   </si>
   <si>
     <t xml:space="preserve">Cross-check on Appendix D.3 assessed GCP intensity of 335 (row 17)</t>
   </si>
   <si>
-    <t xml:space="preserve">Google realised market-based intensity, CY2024 (gCO2e/kWh)</t>
+    <t xml:space="preserve">Google realized market-based intensity, CY2024 (gCO2e/kWh)</t>
   </si>
   <si>
     <t xml:space="preserve">Prior-year comparator only</t>
@@ -327,7 +327,7 @@
     <t xml:space="preserve">Procurement-lag row credits Oracle/Stargate at its location-based intensity (319) rather than its reported FY25 market-based Scope 2 (46).</t>
   </si>
   <si>
-    <t xml:space="preserve">GCP excluded row renormalises the Azure / Oracle-Stargate / AWS shares of rows 16 – 18 to sum to 100% (Appendix E.6). Single-provider rows bound Table 10: the floor and ceiling a reader reaches by routing all inference to one provider.</t>
+    <t xml:space="preserve">GCP excluded row renormalizes the Azure / Oracle-Stargate / AWS shares of rows 16 – 18 to sum to 100% (Appendix E.6). Single-provider rows bound Table 10: the floor and ceiling a reader reaches by routing all inference to one provider.</t>
   </si>
   <si>
     <t xml:space="preserve">Measured inputs from the frozen corpus (24 Jun - 22 Aug 2026). All values are measured data (medians / daily-median stats), not editable assumptions.</t>
@@ -1183,7 +1183,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="20">
+  <cellXfs count="16">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -1225,22 +1225,6 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="172" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="170" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="171" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -6451,60 +6435,60 @@
   </cols>
   <sheetData>
     <row r="1" s="1" customFormat="true" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1" s="15" t="s">
+      <c r="A1" s="11" t="s">
         <v>262</v>
       </c>
-      <c r="B1" s="15"/>
-      <c r="C1" s="15"/>
-      <c r="D1" s="15"/>
-      <c r="E1" s="15"/>
-      <c r="F1" s="15"/>
-      <c r="G1" s="15"/>
-      <c r="H1" s="15"/>
-      <c r="I1" s="15"/>
-      <c r="J1" s="15"/>
-      <c r="K1" s="15"/>
-      <c r="L1" s="15"/>
-      <c r="M1" s="15"/>
+      <c r="B1" s="11"/>
+      <c r="C1" s="11"/>
+      <c r="D1" s="11"/>
+      <c r="E1" s="11"/>
+      <c r="F1" s="11"/>
+      <c r="G1" s="11"/>
+      <c r="H1" s="11"/>
+      <c r="I1" s="11"/>
+      <c r="J1" s="11"/>
+      <c r="K1" s="11"/>
+      <c r="L1" s="11"/>
+      <c r="M1" s="11"/>
     </row>
     <row r="2" s="1" customFormat="true" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A2" s="16" t="s">
+      <c r="A2" s="12" t="s">
         <v>176</v>
       </c>
-      <c r="B2" s="16" t="s">
+      <c r="B2" s="12" t="s">
         <v>263</v>
       </c>
-      <c r="C2" s="16" t="s">
+      <c r="C2" s="12" t="s">
         <v>264</v>
       </c>
-      <c r="D2" s="16" t="s">
+      <c r="D2" s="12" t="s">
         <v>265</v>
       </c>
-      <c r="E2" s="16" t="s">
+      <c r="E2" s="12" t="s">
         <v>266</v>
       </c>
-      <c r="F2" s="16" t="s">
+      <c r="F2" s="12" t="s">
         <v>267</v>
       </c>
-      <c r="G2" s="16" t="s">
+      <c r="G2" s="12" t="s">
         <v>268</v>
       </c>
-      <c r="H2" s="16" t="s">
+      <c r="H2" s="12" t="s">
         <v>269</v>
       </c>
-      <c r="I2" s="16" t="s">
+      <c r="I2" s="12" t="s">
         <v>270</v>
       </c>
-      <c r="J2" s="16" t="s">
+      <c r="J2" s="12" t="s">
         <v>271</v>
       </c>
-      <c r="K2" s="16" t="s">
+      <c r="K2" s="12" t="s">
         <v>272</v>
       </c>
-      <c r="L2" s="16" t="s">
+      <c r="L2" s="12" t="s">
         <v>273</v>
       </c>
-      <c r="M2" s="15"/>
+      <c r="M2" s="11"/>
       <c r="N2" s="1" t="s">
         <v>274</v>
       </c>
@@ -6522,55 +6506,55 @@
       </c>
     </row>
     <row r="3" s="1" customFormat="true" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A3" s="15" t="str">
+      <c r="A3" s="11" t="str">
         <f aca="false">Levers!A3</f>
         <v>gpt-4o-mini</v>
       </c>
-      <c r="B3" s="15" t="n">
+      <c r="B3" s="11" t="n">
         <f aca="false">Levers!H3</f>
         <v>4.03997840349841</v>
       </c>
-      <c r="C3" s="15" t="n">
+      <c r="C3" s="11" t="n">
         <f aca="false">EXP(Levers!$G3-Levers!B3)</f>
         <v>1.44765892792026</v>
       </c>
-      <c r="D3" s="15" t="n">
+      <c r="D3" s="11" t="n">
         <f aca="false">EXP(Levers!$G3-Levers!C3)</f>
         <v>4.03997840349841</v>
       </c>
-      <c r="E3" s="15" t="n">
+      <c r="E3" s="11" t="n">
         <f aca="false">EXP(Levers!$G3-Levers!D3)</f>
         <v>3.7261936731296</v>
       </c>
-      <c r="F3" s="15" t="n">
+      <c r="F3" s="11" t="n">
         <f aca="false">EXP(Levers!$G3-Levers!E3)</f>
         <v>3.02570379436965</v>
       </c>
-      <c r="G3" s="15" t="n">
+      <c r="G3" s="11" t="n">
         <f aca="false">EXP(Levers!$G3-Levers!F3)</f>
         <v>4.03997840349841</v>
       </c>
-      <c r="H3" s="15" t="n">
+      <c r="H3" s="11" t="n">
         <f aca="false">B3/C3</f>
         <v>2.79069767441861</v>
       </c>
-      <c r="I3" s="15" t="n">
+      <c r="I3" s="11" t="n">
         <f aca="false">B3/D3</f>
         <v>1</v>
       </c>
-      <c r="J3" s="15" t="n">
+      <c r="J3" s="11" t="n">
         <f aca="false">B3/E3</f>
         <v>1.08421052631579</v>
       </c>
-      <c r="K3" s="15" t="n">
+      <c r="K3" s="11" t="n">
         <f aca="false">B3/F3</f>
         <v>1.33521939953811</v>
       </c>
-      <c r="L3" s="15" t="n">
+      <c r="L3" s="11" t="n">
         <f aca="false">B3/G3</f>
         <v>1</v>
       </c>
-      <c r="M3" s="15"/>
+      <c r="M3" s="11"/>
       <c r="N3" s="9" t="n">
         <f aca="false" t="array" ref="N3:N3">IF(AND(A3&lt;&gt;"gpt-4o-mini",INDEX(Corpus!$Q$3:$Q$60,MATCH(A3,Corpus!$A$3:$A$60,0))&lt;&gt;"None"),1,0)</f>
         <v>0</v>
@@ -6593,55 +6577,55 @@
       </c>
     </row>
     <row r="4" s="1" customFormat="true" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A4" s="15" t="str">
+      <c r="A4" s="11" t="str">
         <f aca="false">Levers!A4</f>
         <v>gpt-5 (non-reasoning)</v>
       </c>
-      <c r="B4" s="15" t="n">
+      <c r="B4" s="11" t="n">
         <f aca="false">Levers!H4</f>
         <v>10.722692855447</v>
       </c>
-      <c r="C4" s="15" t="n">
+      <c r="C4" s="11" t="n">
         <f aca="false">EXP(Levers!$G4-Levers!B4)</f>
         <v>3.84229827320183</v>
       </c>
-      <c r="D4" s="15" t="n">
+      <c r="D4" s="11" t="n">
         <f aca="false">EXP(Levers!$G4-Levers!C4)</f>
         <v>3.83988325228844</v>
       </c>
-      <c r="E4" s="15" t="n">
+      <c r="E4" s="11" t="n">
         <f aca="false">EXP(Levers!$G4-Levers!D4)</f>
         <v>9.88986234240254</v>
       </c>
-      <c r="F4" s="15" t="n">
+      <c r="F4" s="11" t="n">
         <f aca="false">EXP(Levers!$G4-Levers!E4)</f>
         <v>8.44913512390014</v>
       </c>
-      <c r="G4" s="15" t="n">
+      <c r="G4" s="11" t="n">
         <f aca="false">EXP(Levers!$G4-Levers!F4)</f>
         <v>10.722692855447</v>
       </c>
-      <c r="H4" s="15" t="n">
+      <c r="H4" s="11" t="n">
         <f aca="false">B4/C4</f>
         <v>2.7906976744186</v>
       </c>
-      <c r="I4" s="15" t="n">
+      <c r="I4" s="11" t="n">
         <f aca="false">B4/D4</f>
         <v>2.79245283018868</v>
       </c>
-      <c r="J4" s="15" t="n">
+      <c r="J4" s="11" t="n">
         <f aca="false">B4/E4</f>
         <v>1.08421052631579</v>
       </c>
-      <c r="K4" s="15" t="n">
+      <c r="K4" s="11" t="n">
         <f aca="false">B4/F4</f>
         <v>1.26908762828465</v>
       </c>
-      <c r="L4" s="15" t="n">
+      <c r="L4" s="11" t="n">
         <f aca="false">B4/G4</f>
         <v>1</v>
       </c>
-      <c r="M4" s="15"/>
+      <c r="M4" s="11"/>
       <c r="N4" s="9" t="n">
         <f aca="false" t="array" ref="N4:N4">IF(AND(A4&lt;&gt;"gpt-4o-mini",INDEX(Corpus!$Q$3:$Q$60,MATCH(A4,Corpus!$A$3:$A$60,0))&lt;&gt;"None"),1,0)</f>
         <v>0</v>
@@ -6664,55 +6648,55 @@
       </c>
     </row>
     <row r="5" s="1" customFormat="true" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A5" s="15" t="str">
+      <c r="A5" s="11" t="str">
         <f aca="false">Levers!A5</f>
         <v>gpt-5 (low)</v>
       </c>
-      <c r="B5" s="15" t="n">
+      <c r="B5" s="11" t="n">
         <f aca="false">Levers!H5</f>
         <v>11.4583048828245</v>
       </c>
-      <c r="C5" s="15" t="n">
+      <c r="C5" s="11" t="n">
         <f aca="false">EXP(Levers!$G5-Levers!B5)</f>
         <v>4.10589258301212</v>
       </c>
-      <c r="D5" s="15" t="n">
+      <c r="D5" s="11" t="n">
         <f aca="false">EXP(Levers!$G5-Levers!C5)</f>
         <v>4.10331188371419</v>
       </c>
-      <c r="E5" s="15" t="n">
+      <c r="E5" s="11" t="n">
         <f aca="false">EXP(Levers!$G5-Levers!D5)</f>
         <v>10.5683394550323</v>
       </c>
-      <c r="F5" s="15" t="n">
+      <c r="F5" s="11" t="n">
         <f aca="false">EXP(Levers!$G5-Levers!E5)</f>
         <v>8.99735150057685</v>
       </c>
-      <c r="G5" s="15" t="n">
+      <c r="G5" s="11" t="n">
         <f aca="false">EXP(Levers!$G5-Levers!F5)</f>
         <v>10.7601404968587</v>
       </c>
-      <c r="H5" s="15" t="n">
+      <c r="H5" s="11" t="n">
         <f aca="false">B5/C5</f>
         <v>2.79069767441861</v>
       </c>
-      <c r="I5" s="15" t="n">
+      <c r="I5" s="11" t="n">
         <f aca="false">B5/D5</f>
         <v>2.79245283018868</v>
       </c>
-      <c r="J5" s="15" t="n">
+      <c r="J5" s="11" t="n">
         <f aca="false">B5/E5</f>
         <v>1.08421052631579</v>
       </c>
-      <c r="K5" s="15" t="n">
+      <c r="K5" s="11" t="n">
         <f aca="false">B5/F5</f>
         <v>1.27351975546247</v>
       </c>
-      <c r="L5" s="15" t="n">
+      <c r="L5" s="11" t="n">
         <f aca="false">B5/G5</f>
         <v>1.06488431876607</v>
       </c>
-      <c r="M5" s="15"/>
+      <c r="M5" s="11"/>
       <c r="N5" s="9" t="n">
         <f aca="false" t="array" ref="N5:N5">IF(AND(A5&lt;&gt;"gpt-4o-mini",INDEX(Corpus!$Q$3:$Q$60,MATCH(A5,Corpus!$A$3:$A$60,0))&lt;&gt;"None"),1,0)</f>
         <v>1</v>
@@ -6735,55 +6719,55 @@
       </c>
     </row>
     <row r="6" s="1" customFormat="true" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A6" s="15" t="str">
+      <c r="A6" s="11" t="str">
         <f aca="false">Levers!A6</f>
         <v>gpt-5 (medium)</v>
       </c>
-      <c r="B6" s="15" t="n">
+      <c r="B6" s="11" t="n">
         <f aca="false">Levers!H6</f>
         <v>12.6437057548337</v>
       </c>
-      <c r="C6" s="15" t="n">
+      <c r="C6" s="11" t="n">
         <f aca="false">EXP(Levers!$G6-Levers!B6)</f>
         <v>4.53066122881541</v>
       </c>
-      <c r="D6" s="15" t="n">
+      <c r="D6" s="11" t="n">
         <f aca="false">EXP(Levers!$G6-Levers!C6)</f>
         <v>4.5278135473391</v>
       </c>
-      <c r="E6" s="15" t="n">
+      <c r="E6" s="11" t="n">
         <f aca="false">EXP(Levers!$G6-Levers!D6)</f>
         <v>11.6616703564</v>
       </c>
-      <c r="F6" s="15" t="n">
+      <c r="F6" s="11" t="n">
         <f aca="false">EXP(Levers!$G6-Levers!E6)</f>
         <v>9.95807925588682</v>
       </c>
-      <c r="G6" s="15" t="n">
+      <c r="G6" s="11" t="n">
         <f aca="false">EXP(Levers!$G6-Levers!F6)</f>
         <v>10.7278096151194</v>
       </c>
-      <c r="H6" s="15" t="n">
+      <c r="H6" s="11" t="n">
         <f aca="false">B6/C6</f>
         <v>2.79069767441861</v>
       </c>
-      <c r="I6" s="15" t="n">
+      <c r="I6" s="11" t="n">
         <f aca="false">B6/D6</f>
         <v>2.79245283018868</v>
       </c>
-      <c r="J6" s="15" t="n">
+      <c r="J6" s="11" t="n">
         <f aca="false">B6/E6</f>
         <v>1.08421052631579</v>
       </c>
-      <c r="K6" s="15" t="n">
+      <c r="K6" s="11" t="n">
         <f aca="false">B6/F6</f>
         <v>1.26969322395775</v>
       </c>
-      <c r="L6" s="15" t="n">
+      <c r="L6" s="11" t="n">
         <f aca="false">B6/G6</f>
         <v>1.17859154929577</v>
       </c>
-      <c r="M6" s="15"/>
+      <c r="M6" s="11"/>
       <c r="N6" s="9" t="n">
         <f aca="false" t="array" ref="N6:N6">IF(AND(A6&lt;&gt;"gpt-4o-mini",INDEX(Corpus!$Q$3:$Q$60,MATCH(A6,Corpus!$A$3:$A$60,0))&lt;&gt;"None"),1,0)</f>
         <v>1</v>
@@ -6806,55 +6790,55 @@
       </c>
     </row>
     <row r="7" s="1" customFormat="true" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A7" s="15" t="str">
+      <c r="A7" s="11" t="str">
         <f aca="false">Levers!A7</f>
         <v>gpt-5 (high)</v>
       </c>
-      <c r="B7" s="15" t="n">
+      <c r="B7" s="11" t="n">
         <f aca="false">Levers!H7</f>
         <v>11.8695843351047</v>
       </c>
-      <c r="C7" s="15" t="n">
+      <c r="C7" s="11" t="n">
         <f aca="false">EXP(Levers!$G7-Levers!B7)</f>
         <v>4.2532677200792</v>
       </c>
-      <c r="D7" s="15" t="n">
+      <c r="D7" s="11" t="n">
         <f aca="false">EXP(Levers!$G7-Levers!C7)</f>
         <v>4.25059439027399</v>
       </c>
-      <c r="E7" s="15" t="n">
+      <c r="E7" s="11" t="n">
         <f aca="false">EXP(Levers!$G7-Levers!D7)</f>
         <v>10.947674872184</v>
       </c>
-      <c r="F7" s="15" t="n">
+      <c r="F7" s="11" t="n">
         <f aca="false">EXP(Levers!$G7-Levers!E7)</f>
         <v>9.41132369794681</v>
       </c>
-      <c r="G7" s="15" t="n">
+      <c r="G7" s="11" t="n">
         <f aca="false">EXP(Levers!$G7-Levers!F7)</f>
         <v>10.6560697655854</v>
       </c>
-      <c r="H7" s="15" t="n">
+      <c r="H7" s="11" t="n">
         <f aca="false">B7/C7</f>
         <v>2.7906976744186</v>
       </c>
-      <c r="I7" s="15" t="n">
+      <c r="I7" s="11" t="n">
         <f aca="false">B7/D7</f>
         <v>2.79245283018868</v>
       </c>
-      <c r="J7" s="15" t="n">
+      <c r="J7" s="11" t="n">
         <f aca="false">B7/E7</f>
         <v>1.08421052631579</v>
       </c>
-      <c r="K7" s="15" t="n">
+      <c r="K7" s="11" t="n">
         <f aca="false">B7/F7</f>
         <v>1.26120243188471</v>
       </c>
-      <c r="L7" s="15" t="n">
+      <c r="L7" s="11" t="n">
         <f aca="false">B7/G7</f>
         <v>1.11388012618297</v>
       </c>
-      <c r="M7" s="15"/>
+      <c r="M7" s="11"/>
       <c r="N7" s="9" t="n">
         <f aca="false" t="array" ref="N7:N7">IF(AND(A7&lt;&gt;"gpt-4o-mini",INDEX(Corpus!$Q$3:$Q$60,MATCH(A7,Corpus!$A$3:$A$60,0))&lt;&gt;"None"),1,0)</f>
         <v>1</v>
@@ -6877,55 +6861,55 @@
       </c>
     </row>
     <row r="8" s="1" customFormat="true" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A8" s="15" t="str">
+      <c r="A8" s="11" t="str">
         <f aca="false">Levers!A8</f>
         <v>gpt-5 (xhigh)</v>
       </c>
-      <c r="B8" s="15" t="n">
+      <c r="B8" s="11" t="n">
         <f aca="false">Levers!H8</f>
         <v>12.2405736208923</v>
       </c>
-      <c r="C8" s="15" t="n">
+      <c r="C8" s="11" t="n">
         <f aca="false">EXP(Levers!$G8-Levers!B8)</f>
         <v>4.3862055474864</v>
       </c>
-      <c r="D8" s="15" t="n">
+      <c r="D8" s="11" t="n">
         <f aca="false">EXP(Levers!$G8-Levers!C8)</f>
         <v>4.38344866153575</v>
       </c>
-      <c r="E8" s="15" t="n">
+      <c r="E8" s="11" t="n">
         <f aca="false">EXP(Levers!$G8-Levers!D8)</f>
         <v>11.2898494561628</v>
       </c>
-      <c r="F8" s="15" t="n">
+      <c r="F8" s="11" t="n">
         <f aca="false">EXP(Levers!$G8-Levers!E8)</f>
         <v>9.66869954256894</v>
       </c>
-      <c r="G8" s="15" t="n">
+      <c r="G8" s="11" t="n">
         <f aca="false">EXP(Levers!$G8-Levers!F8)</f>
         <v>10.6966050668576</v>
       </c>
-      <c r="H8" s="15" t="n">
+      <c r="H8" s="11" t="n">
         <f aca="false">B8/C8</f>
         <v>2.79069767441861</v>
       </c>
-      <c r="I8" s="15" t="n">
+      <c r="I8" s="11" t="n">
         <f aca="false">B8/D8</f>
         <v>2.79245283018868</v>
       </c>
-      <c r="J8" s="15" t="n">
+      <c r="J8" s="11" t="n">
         <f aca="false">B8/E8</f>
         <v>1.08421052631579</v>
       </c>
-      <c r="K8" s="15" t="n">
+      <c r="K8" s="11" t="n">
         <f aca="false">B8/F8</f>
         <v>1.266</v>
       </c>
-      <c r="L8" s="15" t="n">
+      <c r="L8" s="11" t="n">
         <f aca="false">B8/G8</f>
         <v>1.14434192385195</v>
       </c>
-      <c r="M8" s="15"/>
+      <c r="M8" s="11"/>
       <c r="N8" s="9" t="n">
         <f aca="false" t="array" ref="N8:N8">IF(AND(A8&lt;&gt;"gpt-4o-mini",INDEX(Corpus!$Q$3:$Q$60,MATCH(A8,Corpus!$A$3:$A$60,0))&lt;&gt;"None"),1,0)</f>
         <v>1</v>
@@ -6948,55 +6932,55 @@
       </c>
     </row>
     <row r="9" s="1" customFormat="true" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A9" s="15" t="str">
+      <c r="A9" s="11" t="str">
         <f aca="false">Levers!A9</f>
         <v>gpt-5.2 (non-reasoning)</v>
       </c>
-      <c r="B9" s="15" t="n">
+      <c r="B9" s="11" t="n">
         <f aca="false">Levers!H9</f>
         <v>10.4829226736522</v>
       </c>
-      <c r="C9" s="15" t="n">
+      <c r="C9" s="11" t="n">
         <f aca="false">EXP(Levers!$G9-Levers!B9)</f>
         <v>3.75638062472538</v>
       </c>
-      <c r="D9" s="15" t="n">
+      <c r="D9" s="11" t="n">
         <f aca="false">EXP(Levers!$G9-Levers!C9)</f>
         <v>3.75401960610519</v>
       </c>
-      <c r="E9" s="15" t="n">
+      <c r="E9" s="11" t="n">
         <f aca="false">EXP(Levers!$G9-Levers!D9)</f>
         <v>9.66871508734915</v>
       </c>
-      <c r="F9" s="15" t="n">
+      <c r="F9" s="11" t="n">
         <f aca="false">EXP(Levers!$G9-Levers!E9)</f>
         <v>8.44913512390014</v>
       </c>
-      <c r="G9" s="15" t="n">
+      <c r="G9" s="11" t="n">
         <f aca="false">EXP(Levers!$G9-Levers!F9)</f>
         <v>10.4829226736522</v>
       </c>
-      <c r="H9" s="15" t="n">
+      <c r="H9" s="11" t="n">
         <f aca="false">B9/C9</f>
         <v>2.7906976744186</v>
       </c>
-      <c r="I9" s="15" t="n">
+      <c r="I9" s="11" t="n">
         <f aca="false">B9/D9</f>
         <v>2.79245283018868</v>
       </c>
-      <c r="J9" s="15" t="n">
+      <c r="J9" s="11" t="n">
         <f aca="false">B9/E9</f>
         <v>1.08421052631579</v>
       </c>
-      <c r="K9" s="15" t="n">
+      <c r="K9" s="11" t="n">
         <f aca="false">B9/F9</f>
         <v>1.24070955428315</v>
       </c>
-      <c r="L9" s="15" t="n">
+      <c r="L9" s="11" t="n">
         <f aca="false">B9/G9</f>
         <v>1</v>
       </c>
-      <c r="M9" s="15"/>
+      <c r="M9" s="11"/>
       <c r="N9" s="9" t="n">
         <f aca="false" t="array" ref="N9:N9">IF(AND(A9&lt;&gt;"gpt-4o-mini",INDEX(Corpus!$Q$3:$Q$60,MATCH(A9,Corpus!$A$3:$A$60,0))&lt;&gt;"None"),1,0)</f>
         <v>0</v>
@@ -7019,55 +7003,55 @@
       </c>
     </row>
     <row r="10" s="1" customFormat="true" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A10" s="15" t="str">
+      <c r="A10" s="11" t="str">
         <f aca="false">Levers!A10</f>
         <v>gpt-5.2 (low)</v>
       </c>
-      <c r="B10" s="15" t="n">
+      <c r="B10" s="11" t="n">
         <f aca="false">Levers!H10</f>
         <v>11.0843005102309</v>
       </c>
-      <c r="C10" s="15" t="n">
+      <c r="C10" s="11" t="n">
         <f aca="false">EXP(Levers!$G10-Levers!B10)</f>
         <v>3.97187434949939</v>
       </c>
-      <c r="D10" s="15" t="n">
+      <c r="D10" s="11" t="n">
         <f aca="false">EXP(Levers!$G10-Levers!C10)</f>
         <v>3.96937788542051</v>
       </c>
-      <c r="E10" s="15" t="n">
+      <c r="E10" s="11" t="n">
         <f aca="false">EXP(Levers!$G10-Levers!D10)</f>
         <v>10.2233839657469</v>
       </c>
-      <c r="F10" s="15" t="n">
+      <c r="F10" s="11" t="n">
         <f aca="false">EXP(Levers!$G10-Levers!E10)</f>
         <v>8.91483548505999</v>
       </c>
-      <c r="G10" s="15" t="n">
+      <c r="G10" s="11" t="n">
         <f aca="false">EXP(Levers!$G10-Levers!F10)</f>
         <v>10.5052698865621</v>
       </c>
-      <c r="H10" s="15" t="n">
+      <c r="H10" s="11" t="n">
         <f aca="false">B10/C10</f>
         <v>2.7906976744186</v>
       </c>
-      <c r="I10" s="15" t="n">
+      <c r="I10" s="11" t="n">
         <f aca="false">B10/D10</f>
         <v>2.79245283018868</v>
       </c>
-      <c r="J10" s="15" t="n">
+      <c r="J10" s="11" t="n">
         <f aca="false">B10/E10</f>
         <v>1.08421052631579</v>
       </c>
-      <c r="K10" s="15" t="n">
+      <c r="K10" s="11" t="n">
         <f aca="false">B10/F10</f>
         <v>1.24335446557669</v>
       </c>
-      <c r="L10" s="15" t="n">
+      <c r="L10" s="11" t="n">
         <f aca="false">B10/G10</f>
         <v>1.05511811023622</v>
       </c>
-      <c r="M10" s="15"/>
+      <c r="M10" s="11"/>
       <c r="N10" s="9" t="n">
         <f aca="false" t="array" ref="N10:N10">IF(AND(A10&lt;&gt;"gpt-4o-mini",INDEX(Corpus!$Q$3:$Q$60,MATCH(A10,Corpus!$A$3:$A$60,0))&lt;&gt;"None"),1,0)</f>
         <v>1</v>
@@ -7090,55 +7074,55 @@
       </c>
     </row>
     <row r="11" s="1" customFormat="true" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A11" s="15" t="str">
+      <c r="A11" s="11" t="str">
         <f aca="false">Levers!A11</f>
         <v>gpt-5.2 (medium)</v>
       </c>
-      <c r="B11" s="15" t="n">
+      <c r="B11" s="11" t="n">
         <f aca="false">Levers!H11</f>
         <v>10.8050698350722</v>
       </c>
-      <c r="C11" s="15" t="n">
+      <c r="C11" s="11" t="n">
         <f aca="false">EXP(Levers!$G11-Levers!B11)</f>
         <v>3.87181669090089</v>
       </c>
-      <c r="D11" s="15" t="n">
+      <c r="D11" s="11" t="n">
         <f aca="false">EXP(Levers!$G11-Levers!C11)</f>
         <v>3.86938311661371</v>
       </c>
-      <c r="E11" s="15" t="n">
+      <c r="E11" s="11" t="n">
         <f aca="false">EXP(Levers!$G11-Levers!D11)</f>
         <v>9.96584111001809</v>
       </c>
-      <c r="F11" s="15" t="n">
+      <c r="F11" s="11" t="n">
         <f aca="false">EXP(Levers!$G11-Levers!E11)</f>
         <v>8.72825373695844</v>
       </c>
-      <c r="G11" s="15" t="n">
+      <c r="G11" s="11" t="n">
         <f aca="false">EXP(Levers!$G11-Levers!F11)</f>
         <v>10.4595372466241</v>
       </c>
-      <c r="H11" s="15" t="n">
+      <c r="H11" s="11" t="n">
         <f aca="false">B11/C11</f>
         <v>2.79069767441861</v>
       </c>
-      <c r="I11" s="15" t="n">
+      <c r="I11" s="11" t="n">
         <f aca="false">B11/D11</f>
         <v>2.79245283018868</v>
       </c>
-      <c r="J11" s="15" t="n">
+      <c r="J11" s="11" t="n">
         <f aca="false">B11/E11</f>
         <v>1.08421052631579</v>
       </c>
-      <c r="K11" s="15" t="n">
+      <c r="K11" s="11" t="n">
         <f aca="false">B11/F11</f>
         <v>1.23794176483663</v>
       </c>
-      <c r="L11" s="15" t="n">
+      <c r="L11" s="11" t="n">
         <f aca="false">B11/G11</f>
         <v>1.03303516974995</v>
       </c>
-      <c r="M11" s="15"/>
+      <c r="M11" s="11"/>
       <c r="N11" s="9" t="n">
         <f aca="false" t="array" ref="N11:N11">IF(AND(A11&lt;&gt;"gpt-4o-mini",INDEX(Corpus!$Q$3:$Q$60,MATCH(A11,Corpus!$A$3:$A$60,0))&lt;&gt;"None"),1,0)</f>
         <v>1</v>
@@ -7161,55 +7145,55 @@
       </c>
     </row>
     <row r="12" s="1" customFormat="true" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A12" s="15" t="str">
+      <c r="A12" s="11" t="str">
         <f aca="false">Levers!A12</f>
         <v>gpt-5.2 (high)</v>
       </c>
-      <c r="B12" s="15" t="n">
+      <c r="B12" s="11" t="n">
         <f aca="false">Levers!H12</f>
         <v>10.8050182163209</v>
       </c>
-      <c r="C12" s="15" t="n">
+      <c r="C12" s="11" t="n">
         <f aca="false">EXP(Levers!$G12-Levers!B12)</f>
         <v>3.87179819418165</v>
       </c>
-      <c r="D12" s="15" t="n">
+      <c r="D12" s="11" t="n">
         <f aca="false">EXP(Levers!$G12-Levers!C12)</f>
         <v>3.86936463152032</v>
       </c>
-      <c r="E12" s="15" t="n">
+      <c r="E12" s="11" t="n">
         <f aca="false">EXP(Levers!$G12-Levers!D12)</f>
         <v>9.96579350049014</v>
       </c>
-      <c r="F12" s="15" t="n">
+      <c r="F12" s="11" t="n">
         <f aca="false">EXP(Levers!$G12-Levers!E12)</f>
         <v>8.82753304775717</v>
       </c>
-      <c r="G12" s="15" t="n">
+      <c r="G12" s="11" t="n">
         <f aca="false">EXP(Levers!$G12-Levers!F12)</f>
         <v>10.3418541094097</v>
       </c>
-      <c r="H12" s="15" t="n">
+      <c r="H12" s="11" t="n">
         <f aca="false">B12/C12</f>
         <v>2.7906976744186</v>
       </c>
-      <c r="I12" s="15" t="n">
+      <c r="I12" s="11" t="n">
         <f aca="false">B12/D12</f>
         <v>2.79245283018868</v>
       </c>
-      <c r="J12" s="15" t="n">
+      <c r="J12" s="11" t="n">
         <f aca="false">B12/E12</f>
         <v>1.08421052631579</v>
       </c>
-      <c r="K12" s="15" t="n">
+      <c r="K12" s="11" t="n">
         <f aca="false">B12/F12</f>
         <v>1.22401334074486</v>
       </c>
-      <c r="L12" s="15" t="n">
+      <c r="L12" s="11" t="n">
         <f aca="false">B12/G12</f>
         <v>1.04478540327597</v>
       </c>
-      <c r="M12" s="15"/>
+      <c r="M12" s="11"/>
       <c r="N12" s="9" t="n">
         <f aca="false" t="array" ref="N12:N12">IF(AND(A12&lt;&gt;"gpt-4o-mini",INDEX(Corpus!$Q$3:$Q$60,MATCH(A12,Corpus!$A$3:$A$60,0))&lt;&gt;"None"),1,0)</f>
         <v>1</v>
@@ -7232,55 +7216,55 @@
       </c>
     </row>
     <row r="13" s="1" customFormat="true" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A13" s="15" t="str">
+      <c r="A13" s="11" t="str">
         <f aca="false">Levers!A13</f>
         <v>gpt-5.2 (xhigh)</v>
       </c>
-      <c r="B13" s="15" t="n">
+      <c r="B13" s="11" t="n">
         <f aca="false">Levers!H13</f>
         <v>11.5460522983444</v>
       </c>
-      <c r="C13" s="15" t="n">
+      <c r="C13" s="11" t="n">
         <f aca="false">EXP(Levers!$G13-Levers!B13)</f>
         <v>4.13733540690674</v>
       </c>
-      <c r="D13" s="15" t="n">
+      <c r="D13" s="11" t="n">
         <f aca="false">EXP(Levers!$G13-Levers!C13)</f>
         <v>4.13473494467738</v>
       </c>
-      <c r="E13" s="15" t="n">
+      <c r="E13" s="11" t="n">
         <f aca="false">EXP(Levers!$G13-Levers!D13)</f>
         <v>10.6492715373079</v>
       </c>
-      <c r="F13" s="15" t="n">
+      <c r="F13" s="11" t="n">
         <f aca="false">EXP(Levers!$G13-Levers!E13)</f>
         <v>9.32705022147414</v>
       </c>
-      <c r="G13" s="15" t="n">
+      <c r="G13" s="11" t="n">
         <f aca="false">EXP(Levers!$G13-Levers!F13)</f>
         <v>10.4592720849434</v>
       </c>
-      <c r="H13" s="15" t="n">
+      <c r="H13" s="11" t="n">
         <f aca="false">B13/C13</f>
         <v>2.7906976744186</v>
       </c>
-      <c r="I13" s="15" t="n">
+      <c r="I13" s="11" t="n">
         <f aca="false">B13/D13</f>
         <v>2.79245283018868</v>
       </c>
-      <c r="J13" s="15" t="n">
+      <c r="J13" s="11" t="n">
         <f aca="false">B13/E13</f>
         <v>1.08421052631579</v>
       </c>
-      <c r="K13" s="15" t="n">
+      <c r="K13" s="11" t="n">
         <f aca="false">B13/F13</f>
         <v>1.23791038154392</v>
       </c>
-      <c r="L13" s="15" t="n">
+      <c r="L13" s="11" t="n">
         <f aca="false">B13/G13</f>
         <v>1.1039059128183</v>
       </c>
-      <c r="M13" s="15"/>
+      <c r="M13" s="11"/>
       <c r="N13" s="9" t="n">
         <f aca="false" t="array" ref="N13:N13">IF(AND(A13&lt;&gt;"gpt-4o-mini",INDEX(Corpus!$Q$3:$Q$60,MATCH(A13,Corpus!$A$3:$A$60,0))&lt;&gt;"None"),1,0)</f>
         <v>1</v>
@@ -7303,55 +7287,55 @@
       </c>
     </row>
     <row r="14" s="1" customFormat="true" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A14" s="15" t="str">
+      <c r="A14" s="11" t="str">
         <f aca="false">Levers!A14</f>
         <v>gpt-5.4-nano (non-reasoning)</v>
       </c>
-      <c r="B14" s="15" t="n">
+      <c r="B14" s="11" t="n">
         <f aca="false">Levers!H14</f>
         <v>10.5590492798124</v>
       </c>
-      <c r="C14" s="15" t="n">
+      <c r="C14" s="11" t="n">
         <f aca="false">EXP(Levers!$G14-Levers!B14)</f>
         <v>3.7836593252661</v>
       </c>
-      <c r="D14" s="15" t="n">
+      <c r="D14" s="11" t="n">
         <f aca="false">EXP(Levers!$G14-Levers!C14)</f>
         <v>3.78128116101389</v>
       </c>
-      <c r="E14" s="15" t="n">
+      <c r="E14" s="11" t="n">
         <f aca="false">EXP(Levers!$G14-Levers!D14)</f>
         <v>9.73892894739977</v>
       </c>
-      <c r="F14" s="15" t="n">
+      <c r="F14" s="11" t="n">
         <f aca="false">EXP(Levers!$G14-Levers!E14)</f>
         <v>8.44913512390014</v>
       </c>
-      <c r="G14" s="15" t="n">
+      <c r="G14" s="11" t="n">
         <f aca="false">EXP(Levers!$G14-Levers!F14)</f>
         <v>10.5590492798124</v>
       </c>
-      <c r="H14" s="15" t="n">
+      <c r="H14" s="11" t="n">
         <f aca="false">B14/C14</f>
         <v>2.7906976744186</v>
       </c>
-      <c r="I14" s="15" t="n">
+      <c r="I14" s="11" t="n">
         <f aca="false">B14/D14</f>
         <v>2.79245283018868</v>
       </c>
-      <c r="J14" s="15" t="n">
+      <c r="J14" s="11" t="n">
         <f aca="false">B14/E14</f>
         <v>1.08421052631579</v>
       </c>
-      <c r="K14" s="15" t="n">
+      <c r="K14" s="11" t="n">
         <f aca="false">B14/F14</f>
         <v>1.24971954229302</v>
       </c>
-      <c r="L14" s="15" t="n">
+      <c r="L14" s="11" t="n">
         <f aca="false">B14/G14</f>
         <v>1</v>
       </c>
-      <c r="M14" s="15"/>
+      <c r="M14" s="11"/>
       <c r="N14" s="9" t="n">
         <f aca="false" t="array" ref="N14:N14">IF(AND(A14&lt;&gt;"gpt-4o-mini",INDEX(Corpus!$Q$3:$Q$60,MATCH(A14,Corpus!$A$3:$A$60,0))&lt;&gt;"None"),1,0)</f>
         <v>0</v>
@@ -7374,55 +7358,55 @@
       </c>
     </row>
     <row r="15" s="1" customFormat="true" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A15" s="15" t="str">
+      <c r="A15" s="11" t="str">
         <f aca="false">Levers!A15</f>
         <v>gpt-5.4-nano (low)</v>
       </c>
-      <c r="B15" s="15" t="n">
+      <c r="B15" s="11" t="n">
         <f aca="false">Levers!H15</f>
         <v>10.9334418503663</v>
       </c>
-      <c r="C15" s="15" t="n">
+      <c r="C15" s="11" t="n">
         <f aca="false">EXP(Levers!$G15-Levers!B15)</f>
         <v>3.91781666304792</v>
       </c>
-      <c r="D15" s="15" t="n">
+      <c r="D15" s="11" t="n">
         <f aca="false">EXP(Levers!$G15-Levers!C15)</f>
         <v>3.91535417614468</v>
       </c>
-      <c r="E15" s="15" t="n">
+      <c r="E15" s="11" t="n">
         <f aca="false">EXP(Levers!$G15-Levers!D15)</f>
         <v>10.0842424833475</v>
       </c>
-      <c r="F15" s="15" t="n">
+      <c r="F15" s="11" t="n">
         <f aca="false">EXP(Levers!$G15-Levers!E15)</f>
         <v>8.70550617044308</v>
       </c>
-      <c r="G15" s="15" t="n">
+      <c r="G15" s="11" t="n">
         <f aca="false">EXP(Levers!$G15-Levers!F15)</f>
         <v>10.6114596617818</v>
       </c>
-      <c r="H15" s="15" t="n">
+      <c r="H15" s="11" t="n">
         <f aca="false">B15/C15</f>
         <v>2.79069767441861</v>
       </c>
-      <c r="I15" s="15" t="n">
+      <c r="I15" s="11" t="n">
         <f aca="false">B15/D15</f>
         <v>2.79245283018868</v>
       </c>
-      <c r="J15" s="15" t="n">
+      <c r="J15" s="11" t="n">
         <f aca="false">B15/E15</f>
         <v>1.08421052631579</v>
       </c>
-      <c r="K15" s="15" t="n">
+      <c r="K15" s="11" t="n">
         <f aca="false">B15/F15</f>
         <v>1.25592258925592</v>
       </c>
-      <c r="L15" s="15" t="n">
+      <c r="L15" s="11" t="n">
         <f aca="false">B15/G15</f>
         <v>1.03034287448164</v>
       </c>
-      <c r="M15" s="15"/>
+      <c r="M15" s="11"/>
       <c r="N15" s="9" t="n">
         <f aca="false" t="array" ref="N15:N15">IF(AND(A15&lt;&gt;"gpt-4o-mini",INDEX(Corpus!$Q$3:$Q$60,MATCH(A15,Corpus!$A$3:$A$60,0))&lt;&gt;"None"),1,0)</f>
         <v>1</v>
@@ -7445,55 +7429,55 @@
       </c>
     </row>
     <row r="16" s="1" customFormat="true" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A16" s="15" t="str">
+      <c r="A16" s="11" t="str">
         <f aca="false">Levers!A16</f>
         <v>gpt-5.4-nano (medium)</v>
       </c>
-      <c r="B16" s="15" t="n">
+      <c r="B16" s="11" t="n">
         <f aca="false">Levers!H16</f>
         <v>10.7614493607393</v>
       </c>
-      <c r="C16" s="15" t="n">
+      <c r="C16" s="11" t="n">
         <f aca="false">EXP(Levers!$G16-Levers!B16)</f>
         <v>3.85618602093157</v>
       </c>
-      <c r="D16" s="15" t="n">
+      <c r="D16" s="11" t="n">
         <f aca="false">EXP(Levers!$G16-Levers!C16)</f>
         <v>3.85376227107555</v>
       </c>
-      <c r="E16" s="15" t="n">
+      <c r="E16" s="11" t="n">
         <f aca="false">EXP(Levers!$G16-Levers!D16)</f>
         <v>9.92560863369155</v>
       </c>
-      <c r="F16" s="15" t="n">
+      <c r="F16" s="11" t="n">
         <f aca="false">EXP(Levers!$G16-Levers!E16)</f>
         <v>8.72536839731834</v>
       </c>
-      <c r="G16" s="15" t="n">
+      <c r="G16" s="11" t="n">
         <f aca="false">EXP(Levers!$G16-Levers!F16)</f>
         <v>10.4207565385823</v>
       </c>
-      <c r="H16" s="15" t="n">
+      <c r="H16" s="11" t="n">
         <f aca="false">B16/C16</f>
         <v>2.7906976744186</v>
       </c>
-      <c r="I16" s="15" t="n">
+      <c r="I16" s="11" t="n">
         <f aca="false">B16/D16</f>
         <v>2.79245283018868</v>
       </c>
-      <c r="J16" s="15" t="n">
+      <c r="J16" s="11" t="n">
         <f aca="false">B16/E16</f>
         <v>1.08421052631579</v>
       </c>
-      <c r="K16" s="15" t="n">
+      <c r="K16" s="11" t="n">
         <f aca="false">B16/F16</f>
         <v>1.23335186214564</v>
       </c>
-      <c r="L16" s="15" t="n">
+      <c r="L16" s="11" t="n">
         <f aca="false">B16/G16</f>
         <v>1.03269367448472</v>
       </c>
-      <c r="M16" s="15"/>
+      <c r="M16" s="11"/>
       <c r="N16" s="9" t="n">
         <f aca="false" t="array" ref="N16:N16">IF(AND(A16&lt;&gt;"gpt-4o-mini",INDEX(Corpus!$Q$3:$Q$60,MATCH(A16,Corpus!$A$3:$A$60,0))&lt;&gt;"None"),1,0)</f>
         <v>1</v>
@@ -7516,55 +7500,55 @@
       </c>
     </row>
     <row r="17" s="1" customFormat="true" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A17" s="15" t="str">
+      <c r="A17" s="11" t="str">
         <f aca="false">Levers!A17</f>
         <v>gpt-5.4-nano (high)</v>
       </c>
-      <c r="B17" s="15" t="n">
+      <c r="B17" s="11" t="n">
         <f aca="false">Levers!H17</f>
         <v>11.2755077842756</v>
       </c>
-      <c r="C17" s="15" t="n">
+      <c r="C17" s="11" t="n">
         <f aca="false">EXP(Levers!$G17-Levers!B17)</f>
         <v>4.04039028936541</v>
       </c>
-      <c r="D17" s="15" t="n">
+      <c r="D17" s="11" t="n">
         <f aca="false">EXP(Levers!$G17-Levers!C17)</f>
         <v>4.03785076058517</v>
       </c>
-      <c r="E17" s="15" t="n">
+      <c r="E17" s="11" t="n">
         <f aca="false">EXP(Levers!$G17-Levers!D17)</f>
         <v>10.3997401893804</v>
       </c>
-      <c r="F17" s="15" t="n">
+      <c r="F17" s="11" t="n">
         <f aca="false">EXP(Levers!$G17-Levers!E17)</f>
         <v>8.9526738545123</v>
       </c>
-      <c r="G17" s="15" t="n">
+      <c r="G17" s="11" t="n">
         <f aca="false">EXP(Levers!$G17-Levers!F17)</f>
         <v>10.6413224035762</v>
       </c>
-      <c r="H17" s="15" t="n">
+      <c r="H17" s="11" t="n">
         <f aca="false">B17/C17</f>
         <v>2.7906976744186</v>
       </c>
-      <c r="I17" s="15" t="n">
+      <c r="I17" s="11" t="n">
         <f aca="false">B17/D17</f>
         <v>2.79245283018868</v>
       </c>
-      <c r="J17" s="15" t="n">
+      <c r="J17" s="11" t="n">
         <f aca="false">B17/E17</f>
         <v>1.08421052631579</v>
       </c>
-      <c r="K17" s="15" t="n">
+      <c r="K17" s="11" t="n">
         <f aca="false">B17/F17</f>
         <v>1.25945700329433</v>
       </c>
-      <c r="L17" s="15" t="n">
+      <c r="L17" s="11" t="n">
         <f aca="false">B17/G17</f>
         <v>1.0595964821521</v>
       </c>
-      <c r="M17" s="15"/>
+      <c r="M17" s="11"/>
       <c r="N17" s="9" t="n">
         <f aca="false" t="array" ref="N17:N17">IF(AND(A17&lt;&gt;"gpt-4o-mini",INDEX(Corpus!$Q$3:$Q$60,MATCH(A17,Corpus!$A$3:$A$60,0))&lt;&gt;"None"),1,0)</f>
         <v>1</v>
@@ -7587,55 +7571,55 @@
       </c>
     </row>
     <row r="18" s="1" customFormat="true" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A18" s="15" t="str">
+      <c r="A18" s="11" t="str">
         <f aca="false">Levers!A18</f>
         <v>gpt-5.4-nano (xhigh)</v>
       </c>
-      <c r="B18" s="15" t="n">
+      <c r="B18" s="11" t="n">
         <f aca="false">Levers!H18</f>
         <v>11.4331147319805</v>
       </c>
-      <c r="C18" s="15" t="n">
+      <c r="C18" s="11" t="n">
         <f aca="false">EXP(Levers!$G18-Levers!B18)</f>
         <v>4.09686611229301</v>
       </c>
-      <c r="D18" s="15" t="n">
+      <c r="D18" s="11" t="n">
         <f aca="false">EXP(Levers!$G18-Levers!C18)</f>
         <v>4.09429108645248</v>
       </c>
-      <c r="E18" s="15" t="n">
+      <c r="E18" s="11" t="n">
         <f aca="false">EXP(Levers!$G18-Levers!D18)</f>
         <v>10.5451058207587</v>
       </c>
-      <c r="F18" s="15" t="n">
+      <c r="F18" s="11" t="n">
         <f aca="false">EXP(Levers!$G18-Levers!E18)</f>
         <v>9.0064821990803</v>
       </c>
-      <c r="G18" s="15" t="n">
+      <c r="G18" s="11" t="n">
         <f aca="false">EXP(Levers!$G18-Levers!F18)</f>
         <v>10.7256006421043</v>
       </c>
-      <c r="H18" s="15" t="n">
+      <c r="H18" s="11" t="n">
         <f aca="false">B18/C18</f>
         <v>2.79069767441861</v>
       </c>
-      <c r="I18" s="15" t="n">
+      <c r="I18" s="11" t="n">
         <f aca="false">B18/D18</f>
         <v>2.79245283018868</v>
       </c>
-      <c r="J18" s="15" t="n">
+      <c r="J18" s="11" t="n">
         <f aca="false">B18/E18</f>
         <v>1.08421052631579</v>
       </c>
-      <c r="K18" s="15" t="n">
+      <c r="K18" s="11" t="n">
         <f aca="false">B18/F18</f>
         <v>1.26943178027355</v>
       </c>
-      <c r="L18" s="15" t="n">
+      <c r="L18" s="11" t="n">
         <f aca="false">B18/G18</f>
         <v>1.06596498541059</v>
       </c>
-      <c r="M18" s="15"/>
+      <c r="M18" s="11"/>
       <c r="N18" s="9" t="n">
         <f aca="false" t="array" ref="N18:N18">IF(AND(A18&lt;&gt;"gpt-4o-mini",INDEX(Corpus!$Q$3:$Q$60,MATCH(A18,Corpus!$A$3:$A$60,0))&lt;&gt;"None"),1,0)</f>
         <v>1</v>
@@ -7658,55 +7642,55 @@
       </c>
     </row>
     <row r="19" s="1" customFormat="true" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A19" s="15" t="str">
+      <c r="A19" s="11" t="str">
         <f aca="false">Levers!A19</f>
         <v>gpt-5.4-mini (non-reasoning)</v>
       </c>
-      <c r="B19" s="15" t="n">
+      <c r="B19" s="11" t="n">
         <f aca="false">Levers!H19</f>
         <v>10.442254792607</v>
       </c>
-      <c r="C19" s="15" t="n">
+      <c r="C19" s="11" t="n">
         <f aca="false">EXP(Levers!$G19-Levers!B19)</f>
         <v>3.74180796735083</v>
       </c>
-      <c r="D19" s="15" t="n">
+      <c r="D19" s="11" t="n">
         <f aca="false">EXP(Levers!$G19-Levers!C19)</f>
         <v>3.73945610816331</v>
       </c>
-      <c r="E19" s="15" t="n">
+      <c r="E19" s="11" t="n">
         <f aca="false">EXP(Levers!$G19-Levers!D19)</f>
         <v>9.63120587667634</v>
       </c>
-      <c r="F19" s="15" t="n">
+      <c r="F19" s="11" t="n">
         <f aca="false">EXP(Levers!$G19-Levers!E19)</f>
         <v>8.44913512390014</v>
       </c>
-      <c r="G19" s="15" t="n">
+      <c r="G19" s="11" t="n">
         <f aca="false">EXP(Levers!$G19-Levers!F19)</f>
         <v>10.442254792607</v>
       </c>
-      <c r="H19" s="15" t="n">
+      <c r="H19" s="11" t="n">
         <f aca="false">B19/C19</f>
         <v>2.7906976744186</v>
       </c>
-      <c r="I19" s="15" t="n">
+      <c r="I19" s="11" t="n">
         <f aca="false">B19/D19</f>
         <v>2.79245283018868</v>
       </c>
-      <c r="J19" s="15" t="n">
+      <c r="J19" s="11" t="n">
         <f aca="false">B19/E19</f>
         <v>1.08421052631579</v>
       </c>
-      <c r="K19" s="15" t="n">
+      <c r="K19" s="11" t="n">
         <f aca="false">B19/F19</f>
         <v>1.23589629464782</v>
       </c>
-      <c r="L19" s="15" t="n">
+      <c r="L19" s="11" t="n">
         <f aca="false">B19/G19</f>
         <v>1</v>
       </c>
-      <c r="M19" s="15"/>
+      <c r="M19" s="11"/>
       <c r="N19" s="9" t="n">
         <f aca="false" t="array" ref="N19:N19">IF(AND(A19&lt;&gt;"gpt-4o-mini",INDEX(Corpus!$Q$3:$Q$60,MATCH(A19,Corpus!$A$3:$A$60,0))&lt;&gt;"None"),1,0)</f>
         <v>0</v>
@@ -7729,55 +7713,55 @@
       </c>
     </row>
     <row r="20" s="1" customFormat="true" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A20" s="15" t="str">
+      <c r="A20" s="11" t="str">
         <f aca="false">Levers!A20</f>
         <v>gpt-5.4-mini (low)</v>
       </c>
-      <c r="B20" s="15" t="n">
+      <c r="B20" s="11" t="n">
         <f aca="false">Levers!H20</f>
         <v>10.8144084271898</v>
       </c>
-      <c r="C20" s="15" t="n">
+      <c r="C20" s="11" t="n">
         <f aca="false">EXP(Levers!$G20-Levers!B20)</f>
         <v>3.87516301974302</v>
       </c>
-      <c r="D20" s="15" t="n">
+      <c r="D20" s="11" t="n">
         <f aca="false">EXP(Levers!$G20-Levers!C20)</f>
         <v>3.87272734216933</v>
       </c>
-      <c r="E20" s="15" t="n">
+      <c r="E20" s="11" t="n">
         <f aca="false">EXP(Levers!$G20-Levers!D20)</f>
         <v>9.97445437459255</v>
       </c>
-      <c r="F20" s="15" t="n">
+      <c r="F20" s="11" t="n">
         <f aca="false">EXP(Levers!$G20-Levers!E20)</f>
         <v>8.78196155086467</v>
       </c>
-      <c r="G20" s="15" t="n">
+      <c r="G20" s="11" t="n">
         <f aca="false">EXP(Levers!$G20-Levers!F20)</f>
         <v>10.4045545584716</v>
       </c>
-      <c r="H20" s="15" t="n">
+      <c r="H20" s="11" t="n">
         <f aca="false">B20/C20</f>
         <v>2.7906976744186</v>
       </c>
-      <c r="I20" s="15" t="n">
+      <c r="I20" s="11" t="n">
         <f aca="false">B20/D20</f>
         <v>2.79245283018868</v>
       </c>
-      <c r="J20" s="15" t="n">
+      <c r="J20" s="11" t="n">
         <f aca="false">B20/E20</f>
         <v>1.08421052631579</v>
       </c>
-      <c r="K20" s="15" t="n">
+      <c r="K20" s="11" t="n">
         <f aca="false">B20/F20</f>
         <v>1.23143427178009</v>
       </c>
-      <c r="L20" s="15" t="n">
+      <c r="L20" s="11" t="n">
         <f aca="false">B20/G20</f>
         <v>1.03939177467089</v>
       </c>
-      <c r="M20" s="15"/>
+      <c r="M20" s="11"/>
       <c r="N20" s="9" t="n">
         <f aca="false" t="array" ref="N20:N20">IF(AND(A20&lt;&gt;"gpt-4o-mini",INDEX(Corpus!$Q$3:$Q$60,MATCH(A20,Corpus!$A$3:$A$60,0))&lt;&gt;"None"),1,0)</f>
         <v>1</v>
@@ -7800,55 +7784,55 @@
       </c>
     </row>
     <row r="21" s="1" customFormat="true" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A21" s="15" t="str">
+      <c r="A21" s="11" t="str">
         <f aca="false">Levers!A21</f>
         <v>gpt-5.4-mini (medium)</v>
       </c>
-      <c r="B21" s="15" t="n">
+      <c r="B21" s="11" t="n">
         <f aca="false">Levers!H21</f>
         <v>11.5603522249334</v>
       </c>
-      <c r="C21" s="15" t="n">
+      <c r="C21" s="11" t="n">
         <f aca="false">EXP(Levers!$G21-Levers!B21)</f>
         <v>4.14245954726779</v>
       </c>
-      <c r="D21" s="15" t="n">
+      <c r="D21" s="11" t="n">
         <f aca="false">EXP(Levers!$G21-Levers!C21)</f>
         <v>4.13985586433425</v>
       </c>
-      <c r="E21" s="15" t="n">
+      <c r="E21" s="11" t="n">
         <f aca="false">EXP(Levers!$G21-Levers!D21)</f>
         <v>10.6624607899871</v>
       </c>
-      <c r="F21" s="15" t="n">
+      <c r="F21" s="11" t="n">
         <f aca="false">EXP(Levers!$G21-Levers!E21)</f>
         <v>9.37300532070202</v>
       </c>
-      <c r="G21" s="15" t="n">
+      <c r="G21" s="11" t="n">
         <f aca="false">EXP(Levers!$G21-Levers!F21)</f>
         <v>10.420881530133</v>
       </c>
-      <c r="H21" s="15" t="n">
+      <c r="H21" s="11" t="n">
         <f aca="false">B21/C21</f>
         <v>2.7906976744186</v>
       </c>
-      <c r="I21" s="15" t="n">
+      <c r="I21" s="11" t="n">
         <f aca="false">B21/D21</f>
         <v>2.79245283018868</v>
       </c>
-      <c r="J21" s="15" t="n">
+      <c r="J21" s="11" t="n">
         <f aca="false">B21/E21</f>
         <v>1.08421052631579</v>
       </c>
-      <c r="K21" s="15" t="n">
+      <c r="K21" s="11" t="n">
         <f aca="false">B21/F21</f>
         <v>1.23336665555926</v>
       </c>
-      <c r="L21" s="15" t="n">
+      <c r="L21" s="11" t="n">
         <f aca="false">B21/G21</f>
         <v>1.1093449427964</v>
       </c>
-      <c r="M21" s="15"/>
+      <c r="M21" s="11"/>
       <c r="N21" s="9" t="n">
         <f aca="false" t="array" ref="N21:N21">IF(AND(A21&lt;&gt;"gpt-4o-mini",INDEX(Corpus!$Q$3:$Q$60,MATCH(A21,Corpus!$A$3:$A$60,0))&lt;&gt;"None"),1,0)</f>
         <v>1</v>
@@ -7871,55 +7855,55 @@
       </c>
     </row>
     <row r="22" s="1" customFormat="true" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A22" s="15" t="str">
+      <c r="A22" s="11" t="str">
         <f aca="false">Levers!A22</f>
         <v>gpt-5.4-mini (high)</v>
       </c>
-      <c r="B22" s="15" t="n">
+      <c r="B22" s="11" t="n">
         <f aca="false">Levers!H22</f>
         <v>11.2133264125455</v>
       </c>
-      <c r="C22" s="15" t="n">
+      <c r="C22" s="11" t="n">
         <f aca="false">EXP(Levers!$G22-Levers!B22)</f>
         <v>4.01810863116213</v>
       </c>
-      <c r="D22" s="15" t="n">
+      <c r="D22" s="11" t="n">
         <f aca="false">EXP(Levers!$G22-Levers!C22)</f>
         <v>4.01558310719534</v>
       </c>
-      <c r="E22" s="15" t="n">
+      <c r="E22" s="11" t="n">
         <f aca="false">EXP(Levers!$G22-Levers!D22)</f>
         <v>10.3423884387555</v>
       </c>
-      <c r="F22" s="15" t="n">
+      <c r="F22" s="11" t="n">
         <f aca="false">EXP(Levers!$G22-Levers!E22)</f>
         <v>9.13106905879891</v>
       </c>
-      <c r="G22" s="15" t="n">
+      <c r="G22" s="11" t="n">
         <f aca="false">EXP(Levers!$G22-Levers!F22)</f>
         <v>10.3758836383675</v>
       </c>
-      <c r="H22" s="15" t="n">
+      <c r="H22" s="11" t="n">
         <f aca="false">B22/C22</f>
         <v>2.7906976744186</v>
       </c>
-      <c r="I22" s="15" t="n">
+      <c r="I22" s="11" t="n">
         <f aca="false">B22/D22</f>
         <v>2.79245283018868</v>
       </c>
-      <c r="J22" s="15" t="n">
+      <c r="J22" s="11" t="n">
         <f aca="false">B22/E22</f>
         <v>1.08421052631579</v>
       </c>
-      <c r="K22" s="15" t="n">
+      <c r="K22" s="11" t="n">
         <f aca="false">B22/F22</f>
         <v>1.22804091616633</v>
       </c>
-      <c r="L22" s="15" t="n">
+      <c r="L22" s="11" t="n">
         <f aca="false">B22/G22</f>
         <v>1.08071050171393</v>
       </c>
-      <c r="M22" s="15"/>
+      <c r="M22" s="11"/>
       <c r="N22" s="9" t="n">
         <f aca="false" t="array" ref="N22:N22">IF(AND(A22&lt;&gt;"gpt-4o-mini",INDEX(Corpus!$Q$3:$Q$60,MATCH(A22,Corpus!$A$3:$A$60,0))&lt;&gt;"None"),1,0)</f>
         <v>1</v>
@@ -7942,55 +7926,55 @@
       </c>
     </row>
     <row r="23" s="1" customFormat="true" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A23" s="15" t="str">
+      <c r="A23" s="11" t="str">
         <f aca="false">Levers!A23</f>
         <v>gpt-5.4-mini (xhigh)</v>
       </c>
-      <c r="B23" s="15" t="n">
+      <c r="B23" s="11" t="n">
         <f aca="false">Levers!H23</f>
         <v>18.8996952581074</v>
       </c>
-      <c r="C23" s="15" t="n">
+      <c r="C23" s="11" t="n">
         <f aca="false">EXP(Levers!$G23-Levers!B23)</f>
         <v>6.77239080082183</v>
       </c>
-      <c r="D23" s="15" t="n">
+      <c r="D23" s="11" t="n">
         <f aca="false">EXP(Levers!$G23-Levers!C23)</f>
         <v>6.76813411270064</v>
       </c>
-      <c r="E23" s="15" t="n">
+      <c r="E23" s="11" t="n">
         <f aca="false">EXP(Levers!$G23-Levers!D23)</f>
         <v>17.4317577623321</v>
       </c>
-      <c r="F23" s="15" t="n">
+      <c r="F23" s="11" t="n">
         <f aca="false">EXP(Levers!$G23-Levers!E23)</f>
         <v>13.6115328598181</v>
       </c>
-      <c r="G23" s="15" t="n">
+      <c r="G23" s="11" t="n">
         <f aca="false">EXP(Levers!$G23-Levers!F23)</f>
         <v>11.7316749465951</v>
       </c>
-      <c r="H23" s="15" t="n">
+      <c r="H23" s="11" t="n">
         <f aca="false">B23/C23</f>
         <v>2.7906976744186</v>
       </c>
-      <c r="I23" s="15" t="n">
+      <c r="I23" s="11" t="n">
         <f aca="false">B23/D23</f>
         <v>2.79245283018868</v>
       </c>
-      <c r="J23" s="15" t="n">
+      <c r="J23" s="11" t="n">
         <f aca="false">B23/E23</f>
         <v>1.08421052631579</v>
       </c>
-      <c r="K23" s="15" t="n">
+      <c r="K23" s="11" t="n">
         <f aca="false">B23/F23</f>
         <v>1.38850601565238</v>
       </c>
-      <c r="L23" s="15" t="n">
+      <c r="L23" s="11" t="n">
         <f aca="false">B23/G23</f>
         <v>1.6109971802102</v>
       </c>
-      <c r="M23" s="15"/>
+      <c r="M23" s="11"/>
       <c r="N23" s="9" t="n">
         <f aca="false" t="array" ref="N23:N23">IF(AND(A23&lt;&gt;"gpt-4o-mini",INDEX(Corpus!$Q$3:$Q$60,MATCH(A23,Corpus!$A$3:$A$60,0))&lt;&gt;"None"),1,0)</f>
         <v>1</v>
@@ -8013,55 +7997,55 @@
       </c>
     </row>
     <row r="24" s="1" customFormat="true" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A24" s="15" t="str">
+      <c r="A24" s="11" t="str">
         <f aca="false">Levers!A24</f>
         <v>gpt-5.4 (non-reasoning)</v>
       </c>
-      <c r="B24" s="15" t="n">
+      <c r="B24" s="11" t="n">
         <f aca="false">Levers!H24</f>
         <v>10.6746825264006</v>
       </c>
-      <c r="C24" s="15" t="n">
+      <c r="C24" s="11" t="n">
         <f aca="false">EXP(Levers!$G24-Levers!B24)</f>
         <v>3.82509457196023</v>
       </c>
-      <c r="D24" s="15" t="n">
+      <c r="D24" s="11" t="n">
         <f aca="false">EXP(Levers!$G24-Levers!C24)</f>
         <v>3.82269036418402</v>
       </c>
-      <c r="E24" s="15" t="n">
+      <c r="E24" s="11" t="n">
         <f aca="false">EXP(Levers!$G24-Levers!D24)</f>
         <v>9.84558097095205</v>
       </c>
-      <c r="F24" s="15" t="n">
+      <c r="F24" s="11" t="n">
         <f aca="false">EXP(Levers!$G24-Levers!E24)</f>
         <v>8.44913512390014</v>
       </c>
-      <c r="G24" s="15" t="n">
+      <c r="G24" s="11" t="n">
         <f aca="false">EXP(Levers!$G24-Levers!F24)</f>
         <v>10.6746825264006</v>
       </c>
-      <c r="H24" s="15" t="n">
+      <c r="H24" s="11" t="n">
         <f aca="false">B24/C24</f>
         <v>2.7906976744186</v>
       </c>
-      <c r="I24" s="15" t="n">
+      <c r="I24" s="11" t="n">
         <f aca="false">B24/D24</f>
         <v>2.79245283018868</v>
       </c>
-      <c r="J24" s="15" t="n">
+      <c r="J24" s="11" t="n">
         <f aca="false">B24/E24</f>
         <v>1.08421052631579</v>
       </c>
-      <c r="K24" s="15" t="n">
+      <c r="K24" s="11" t="n">
         <f aca="false">B24/F24</f>
         <v>1.26340535094593</v>
       </c>
-      <c r="L24" s="15" t="n">
+      <c r="L24" s="11" t="n">
         <f aca="false">B24/G24</f>
         <v>1</v>
       </c>
-      <c r="M24" s="15"/>
+      <c r="M24" s="11"/>
       <c r="N24" s="9" t="n">
         <f aca="false" t="array" ref="N24:N24">IF(AND(A24&lt;&gt;"gpt-4o-mini",INDEX(Corpus!$Q$3:$Q$60,MATCH(A24,Corpus!$A$3:$A$60,0))&lt;&gt;"None"),1,0)</f>
         <v>0</v>
@@ -8084,55 +8068,55 @@
       </c>
     </row>
     <row r="25" s="1" customFormat="true" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A25" s="15" t="str">
+      <c r="A25" s="11" t="str">
         <f aca="false">Levers!A25</f>
         <v>gpt-5.4 (low)</v>
       </c>
-      <c r="B25" s="15" t="n">
+      <c r="B25" s="11" t="n">
         <f aca="false">Levers!H25</f>
         <v>10.6736922836178</v>
       </c>
-      <c r="C25" s="15" t="n">
+      <c r="C25" s="11" t="n">
         <f aca="false">EXP(Levers!$G25-Levers!B25)</f>
         <v>3.82473973496303</v>
       </c>
-      <c r="D25" s="15" t="n">
+      <c r="D25" s="11" t="n">
         <f aca="false">EXP(Levers!$G25-Levers!C25)</f>
         <v>3.82233575021447</v>
       </c>
-      <c r="E25" s="15" t="n">
+      <c r="E25" s="11" t="n">
         <f aca="false">EXP(Levers!$G25-Levers!D25)</f>
         <v>9.84466764022997</v>
       </c>
-      <c r="F25" s="15" t="n">
+      <c r="F25" s="11" t="n">
         <f aca="false">EXP(Levers!$G25-Levers!E25)</f>
         <v>8.64005676898777</v>
       </c>
-      <c r="G25" s="15" t="n">
+      <c r="G25" s="11" t="n">
         <f aca="false">EXP(Levers!$G25-Levers!F25)</f>
         <v>10.4378328506958</v>
       </c>
-      <c r="H25" s="15" t="n">
+      <c r="H25" s="11" t="n">
         <f aca="false">B25/C25</f>
         <v>2.79069767441861</v>
       </c>
-      <c r="I25" s="15" t="n">
+      <c r="I25" s="11" t="n">
         <f aca="false">B25/D25</f>
         <v>2.79245283018868</v>
       </c>
-      <c r="J25" s="15" t="n">
+      <c r="J25" s="11" t="n">
         <f aca="false">B25/E25</f>
         <v>1.08421052631579</v>
       </c>
-      <c r="K25" s="15" t="n">
+      <c r="K25" s="11" t="n">
         <f aca="false">B25/F25</f>
         <v>1.23537293434569</v>
       </c>
-      <c r="L25" s="15" t="n">
+      <c r="L25" s="11" t="n">
         <f aca="false">B25/G25</f>
         <v>1.02259659033592</v>
       </c>
-      <c r="M25" s="15"/>
+      <c r="M25" s="11"/>
       <c r="N25" s="9" t="n">
         <f aca="false" t="array" ref="N25:N25">IF(AND(A25&lt;&gt;"gpt-4o-mini",INDEX(Corpus!$Q$3:$Q$60,MATCH(A25,Corpus!$A$3:$A$60,0))&lt;&gt;"None"),1,0)</f>
         <v>1</v>
@@ -8155,55 +8139,55 @@
       </c>
     </row>
     <row r="26" s="1" customFormat="true" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A26" s="15" t="str">
+      <c r="A26" s="11" t="str">
         <f aca="false">Levers!A26</f>
         <v>gpt-5.4 (medium)</v>
       </c>
-      <c r="B26" s="15" t="n">
+      <c r="B26" s="11" t="n">
         <f aca="false">Levers!H26</f>
         <v>11.2620367470057</v>
       </c>
-      <c r="C26" s="15" t="n">
+      <c r="C26" s="11" t="n">
         <f aca="false">EXP(Levers!$G26-Levers!B26)</f>
         <v>4.03556316767705</v>
       </c>
-      <c r="D26" s="15" t="n">
+      <c r="D26" s="11" t="n">
         <f aca="false">EXP(Levers!$G26-Levers!C26)</f>
         <v>4.03302667291421</v>
       </c>
-      <c r="E26" s="15" t="n">
+      <c r="E26" s="11" t="n">
         <f aca="false">EXP(Levers!$G26-Levers!D26)</f>
         <v>10.3873154462674</v>
       </c>
-      <c r="F26" s="15" t="n">
+      <c r="F26" s="11" t="n">
         <f aca="false">EXP(Levers!$G26-Levers!E26)</f>
         <v>8.93873876202607</v>
       </c>
-      <c r="G26" s="15" t="n">
+      <c r="G26" s="11" t="n">
         <f aca="false">EXP(Levers!$G26-Levers!F26)</f>
         <v>10.6451785625529</v>
       </c>
-      <c r="H26" s="15" t="n">
+      <c r="H26" s="11" t="n">
         <f aca="false">B26/C26</f>
         <v>2.79069767441861</v>
       </c>
-      <c r="I26" s="15" t="n">
+      <c r="I26" s="11" t="n">
         <f aca="false">B26/D26</f>
         <v>2.79245283018868</v>
       </c>
-      <c r="J26" s="15" t="n">
+      <c r="J26" s="11" t="n">
         <f aca="false">B26/E26</f>
         <v>1.08421052631579</v>
       </c>
-      <c r="K26" s="15" t="n">
+      <c r="K26" s="11" t="n">
         <f aca="false">B26/F26</f>
         <v>1.25991340018232</v>
       </c>
-      <c r="L26" s="15" t="n">
+      <c r="L26" s="11" t="n">
         <f aca="false">B26/G26</f>
         <v>1.05794718997226</v>
       </c>
-      <c r="M26" s="15"/>
+      <c r="M26" s="11"/>
       <c r="N26" s="9" t="n">
         <f aca="false" t="array" ref="N26:N26">IF(AND(A26&lt;&gt;"gpt-4o-mini",INDEX(Corpus!$Q$3:$Q$60,MATCH(A26,Corpus!$A$3:$A$60,0))&lt;&gt;"None"),1,0)</f>
         <v>1</v>
@@ -8226,55 +8210,55 @@
       </c>
     </row>
     <row r="27" s="1" customFormat="true" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A27" s="15" t="str">
+      <c r="A27" s="11" t="str">
         <f aca="false">Levers!A27</f>
         <v>gpt-5.4 (high)</v>
       </c>
-      <c r="B27" s="15" t="n">
+      <c r="B27" s="11" t="n">
         <f aca="false">Levers!H27</f>
         <v>11.5092719923191</v>
       </c>
-      <c r="C27" s="15" t="n">
+      <c r="C27" s="11" t="n">
         <f aca="false">EXP(Levers!$G27-Levers!B27)</f>
         <v>4.12415579724769</v>
       </c>
-      <c r="D27" s="15" t="n">
+      <c r="D27" s="11" t="n">
         <f aca="false">EXP(Levers!$G27-Levers!C27)</f>
         <v>4.12156361887104</v>
       </c>
-      <c r="E27" s="15" t="n">
+      <c r="E27" s="11" t="n">
         <f aca="false">EXP(Levers!$G27-Levers!D27)</f>
         <v>10.6153479540808</v>
       </c>
-      <c r="F27" s="15" t="n">
+      <c r="F27" s="11" t="n">
         <f aca="false">EXP(Levers!$G27-Levers!E27)</f>
         <v>9.31015466408945</v>
       </c>
-      <c r="G27" s="15" t="n">
+      <c r="G27" s="11" t="n">
         <f aca="false">EXP(Levers!$G27-Levers!F27)</f>
         <v>10.4448741991264</v>
       </c>
-      <c r="H27" s="15" t="n">
+      <c r="H27" s="11" t="n">
         <f aca="false">B27/C27</f>
         <v>2.79069767441861</v>
       </c>
-      <c r="I27" s="15" t="n">
+      <c r="I27" s="11" t="n">
         <f aca="false">B27/D27</f>
         <v>2.79245283018868</v>
       </c>
-      <c r="J27" s="15" t="n">
+      <c r="J27" s="11" t="n">
         <f aca="false">B27/E27</f>
         <v>1.08421052631579</v>
       </c>
-      <c r="K27" s="15" t="n">
+      <c r="K27" s="11" t="n">
         <f aca="false">B27/F27</f>
         <v>1.23620631531633</v>
       </c>
-      <c r="L27" s="15" t="n">
+      <c r="L27" s="11" t="n">
         <f aca="false">B27/G27</f>
         <v>1.10190623390005</v>
       </c>
-      <c r="M27" s="15"/>
+      <c r="M27" s="11"/>
       <c r="N27" s="9" t="n">
         <f aca="false" t="array" ref="N27:N27">IF(AND(A27&lt;&gt;"gpt-4o-mini",INDEX(Corpus!$Q$3:$Q$60,MATCH(A27,Corpus!$A$3:$A$60,0))&lt;&gt;"None"),1,0)</f>
         <v>1</v>
@@ -8297,55 +8281,55 @@
       </c>
     </row>
     <row r="28" s="1" customFormat="true" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A28" s="15" t="str">
+      <c r="A28" s="11" t="str">
         <f aca="false">Levers!A28</f>
         <v>gpt-5.4 (xhigh)</v>
       </c>
-      <c r="B28" s="15" t="n">
+      <c r="B28" s="11" t="n">
         <f aca="false">Levers!H28</f>
         <v>12.1392274803831</v>
       </c>
-      <c r="C28" s="15" t="n">
+      <c r="C28" s="11" t="n">
         <f aca="false">EXP(Levers!$G28-Levers!B28)</f>
         <v>4.34988984713726</v>
       </c>
-      <c r="D28" s="15" t="n">
+      <c r="D28" s="11" t="n">
         <f aca="false">EXP(Levers!$G28-Levers!C28)</f>
         <v>4.34715578689393</v>
       </c>
-      <c r="E28" s="15" t="n">
+      <c r="E28" s="11" t="n">
         <f aca="false">EXP(Levers!$G28-Levers!D28)</f>
         <v>11.1963748605475</v>
       </c>
-      <c r="F28" s="15" t="n">
+      <c r="F28" s="11" t="n">
         <f aca="false">EXP(Levers!$G28-Levers!E28)</f>
         <v>9.7476281447384</v>
       </c>
-      <c r="G28" s="15" t="n">
+      <c r="G28" s="11" t="n">
         <f aca="false">EXP(Levers!$G28-Levers!F28)</f>
         <v>10.522146696464</v>
       </c>
-      <c r="H28" s="15" t="n">
+      <c r="H28" s="11" t="n">
         <f aca="false">B28/C28</f>
         <v>2.7906976744186</v>
       </c>
-      <c r="I28" s="15" t="n">
+      <c r="I28" s="11" t="n">
         <f aca="false">B28/D28</f>
         <v>2.79245283018868</v>
       </c>
-      <c r="J28" s="15" t="n">
+      <c r="J28" s="11" t="n">
         <f aca="false">B28/E28</f>
         <v>1.08421052631579</v>
       </c>
-      <c r="K28" s="15" t="n">
+      <c r="K28" s="11" t="n">
         <f aca="false">B28/F28</f>
         <v>1.24535192563081</v>
       </c>
-      <c r="L28" s="15" t="n">
+      <c r="L28" s="11" t="n">
         <f aca="false">B28/G28</f>
         <v>1.15368354296586</v>
       </c>
-      <c r="M28" s="15"/>
+      <c r="M28" s="11"/>
       <c r="N28" s="9" t="n">
         <f aca="false" t="array" ref="N28:N28">IF(AND(A28&lt;&gt;"gpt-4o-mini",INDEX(Corpus!$Q$3:$Q$60,MATCH(A28,Corpus!$A$3:$A$60,0))&lt;&gt;"None"),1,0)</f>
         <v>1</v>
@@ -8368,55 +8352,55 @@
       </c>
     </row>
     <row r="29" s="1" customFormat="true" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A29" s="15" t="str">
+      <c r="A29" s="11" t="str">
         <f aca="false">Levers!A29</f>
         <v>gpt-5.5 (minimal)</v>
       </c>
-      <c r="B29" s="15" t="n">
+      <c r="B29" s="11" t="n">
         <f aca="false">Levers!H29</f>
         <v>12.2589505268796</v>
       </c>
-      <c r="C29" s="15" t="n">
+      <c r="C29" s="11" t="n">
         <f aca="false">EXP(Levers!$G29-Levers!B29)</f>
         <v>4.39279060546518</v>
       </c>
-      <c r="D29" s="15" t="n">
+      <c r="D29" s="11" t="n">
         <f aca="false">EXP(Levers!$G29-Levers!C29)</f>
         <v>4.39002958057174</v>
       </c>
-      <c r="E29" s="15" t="n">
+      <c r="E29" s="11" t="n">
         <f aca="false">EXP(Levers!$G29-Levers!D29)</f>
         <v>11.3067990296462</v>
       </c>
-      <c r="F29" s="15" t="n">
+      <c r="F29" s="11" t="n">
         <f aca="false">EXP(Levers!$G29-Levers!E29)</f>
         <v>9.79989553208304</v>
       </c>
-      <c r="G29" s="15" t="n">
+      <c r="G29" s="11" t="n">
         <f aca="false">EXP(Levers!$G29-Levers!F29)</f>
         <v>10.5692483292009</v>
       </c>
-      <c r="H29" s="15" t="n">
+      <c r="H29" s="11" t="n">
         <f aca="false">B29/C29</f>
         <v>2.79069767441861</v>
       </c>
-      <c r="I29" s="15" t="n">
+      <c r="I29" s="11" t="n">
         <f aca="false">B29/D29</f>
         <v>2.79245283018868</v>
       </c>
-      <c r="J29" s="15" t="n">
+      <c r="J29" s="11" t="n">
         <f aca="false">B29/E29</f>
         <v>1.08421052631579</v>
       </c>
-      <c r="K29" s="15" t="n">
+      <c r="K29" s="11" t="n">
         <f aca="false">B29/F29</f>
         <v>1.25092665393687</v>
       </c>
-      <c r="L29" s="15" t="n">
+      <c r="L29" s="11" t="n">
         <f aca="false">B29/G29</f>
         <v>1.15986966575573</v>
       </c>
-      <c r="M29" s="15"/>
+      <c r="M29" s="11"/>
       <c r="N29" s="9" t="n">
         <f aca="false" t="array" ref="N29:N29">IF(AND(A29&lt;&gt;"gpt-4o-mini",INDEX(Corpus!$Q$3:$Q$60,MATCH(A29,Corpus!$A$3:$A$60,0))&lt;&gt;"None"),1,0)</f>
         <v>1</v>
@@ -8439,55 +8423,55 @@
       </c>
     </row>
     <row r="30" s="1" customFormat="true" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A30" s="15" t="str">
+      <c r="A30" s="11" t="str">
         <f aca="false">Levers!A30</f>
         <v>gpt-5.5 (low)</v>
       </c>
-      <c r="B30" s="15" t="n">
+      <c r="B30" s="11" t="n">
         <f aca="false">Levers!H30</f>
         <v>10.9374307259003</v>
       </c>
-      <c r="C30" s="15" t="n">
+      <c r="C30" s="11" t="n">
         <f aca="false">EXP(Levers!$G30-Levers!B30)</f>
         <v>3.91924601011429</v>
       </c>
-      <c r="D30" s="15" t="n">
+      <c r="D30" s="11" t="n">
         <f aca="false">EXP(Levers!$G30-Levers!C30)</f>
         <v>3.91678262481566</v>
       </c>
-      <c r="E30" s="15" t="n">
+      <c r="E30" s="11" t="n">
         <f aca="false">EXP(Levers!$G30-Levers!D30)</f>
         <v>10.0879215433061</v>
       </c>
-      <c r="F30" s="15" t="n">
+      <c r="F30" s="11" t="n">
         <f aca="false">EXP(Levers!$G30-Levers!E30)</f>
         <v>8.7665831777977</v>
       </c>
-      <c r="G30" s="15" t="n">
+      <c r="G30" s="11" t="n">
         <f aca="false">EXP(Levers!$G30-Levers!F30)</f>
         <v>10.5413737869358</v>
       </c>
-      <c r="H30" s="15" t="n">
+      <c r="H30" s="11" t="n">
         <f aca="false">B30/C30</f>
         <v>2.7906976744186</v>
       </c>
-      <c r="I30" s="15" t="n">
+      <c r="I30" s="11" t="n">
         <f aca="false">B30/D30</f>
         <v>2.79245283018868</v>
       </c>
-      <c r="J30" s="15" t="n">
+      <c r="J30" s="11" t="n">
         <f aca="false">B30/E30</f>
         <v>1.08421052631579</v>
       </c>
-      <c r="K30" s="15" t="n">
+      <c r="K30" s="11" t="n">
         <f aca="false">B30/F30</f>
         <v>1.24762755386848</v>
       </c>
-      <c r="L30" s="15" t="n">
+      <c r="L30" s="11" t="n">
         <f aca="false">B30/G30</f>
         <v>1.03757166257166</v>
       </c>
-      <c r="M30" s="15"/>
+      <c r="M30" s="11"/>
       <c r="N30" s="9" t="n">
         <f aca="false" t="array" ref="N30:N30">IF(AND(A30&lt;&gt;"gpt-4o-mini",INDEX(Corpus!$Q$3:$Q$60,MATCH(A30,Corpus!$A$3:$A$60,0))&lt;&gt;"None"),1,0)</f>
         <v>1</v>
@@ -8510,55 +8494,55 @@
       </c>
     </row>
     <row r="31" s="1" customFormat="true" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A31" s="15" t="str">
+      <c r="A31" s="11" t="str">
         <f aca="false">Levers!A31</f>
         <v>gpt-5.5 (medium)</v>
       </c>
-      <c r="B31" s="15" t="n">
+      <c r="B31" s="11" t="n">
         <f aca="false">Levers!H31</f>
         <v>12.5841416537109</v>
       </c>
-      <c r="C31" s="15" t="n">
+      <c r="C31" s="11" t="n">
         <f aca="false">EXP(Levers!$G31-Levers!B31)</f>
         <v>4.50931742591307</v>
       </c>
-      <c r="D31" s="15" t="n">
+      <c r="D31" s="11" t="n">
         <f aca="false">EXP(Levers!$G31-Levers!C31)</f>
         <v>4.50648315977485</v>
       </c>
-      <c r="E31" s="15" t="n">
+      <c r="E31" s="11" t="n">
         <f aca="false">EXP(Levers!$G31-Levers!D31)</f>
         <v>11.6067325932285</v>
       </c>
-      <c r="F31" s="15" t="n">
+      <c r="F31" s="11" t="n">
         <f aca="false">EXP(Levers!$G31-Levers!E31)</f>
         <v>10.0586597329788</v>
       </c>
-      <c r="G31" s="15" t="n">
+      <c r="G31" s="11" t="n">
         <f aca="false">EXP(Levers!$G31-Levers!F31)</f>
         <v>10.5705050248296</v>
       </c>
-      <c r="H31" s="15" t="n">
+      <c r="H31" s="11" t="n">
         <f aca="false">B31/C31</f>
         <v>2.79069767441861</v>
       </c>
-      <c r="I31" s="15" t="n">
+      <c r="I31" s="11" t="n">
         <f aca="false">B31/D31</f>
         <v>2.79245283018868</v>
       </c>
-      <c r="J31" s="15" t="n">
+      <c r="J31" s="11" t="n">
         <f aca="false">B31/E31</f>
         <v>1.08421052631579</v>
       </c>
-      <c r="K31" s="15" t="n">
+      <c r="K31" s="11" t="n">
         <f aca="false">B31/F31</f>
         <v>1.25107539053656</v>
       </c>
-      <c r="L31" s="15" t="n">
+      <c r="L31" s="11" t="n">
         <f aca="false">B31/G31</f>
         <v>1.19049578276075</v>
       </c>
-      <c r="M31" s="15"/>
+      <c r="M31" s="11"/>
       <c r="N31" s="9" t="n">
         <f aca="false" t="array" ref="N31:N31">IF(AND(A31&lt;&gt;"gpt-4o-mini",INDEX(Corpus!$Q$3:$Q$60,MATCH(A31,Corpus!$A$3:$A$60,0))&lt;&gt;"None"),1,0)</f>
         <v>1</v>
@@ -8581,55 +8565,55 @@
       </c>
     </row>
     <row r="32" s="1" customFormat="true" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A32" s="15" t="str">
+      <c r="A32" s="11" t="str">
         <f aca="false">Levers!A32</f>
         <v>gpt-5.5 (high)</v>
       </c>
-      <c r="B32" s="15" t="n">
+      <c r="B32" s="11" t="n">
         <f aca="false">Levers!H32</f>
         <v>10.9488957953331</v>
       </c>
-      <c r="C32" s="15" t="n">
+      <c r="C32" s="11" t="n">
         <f aca="false">EXP(Levers!$G32-Levers!B32)</f>
         <v>3.92335432666103</v>
       </c>
-      <c r="D32" s="15" t="n">
+      <c r="D32" s="11" t="n">
         <f aca="false">EXP(Levers!$G32-Levers!C32)</f>
         <v>3.92088835913955</v>
       </c>
-      <c r="E32" s="15" t="n">
+      <c r="E32" s="11" t="n">
         <f aca="false">EXP(Levers!$G32-Levers!D32)</f>
         <v>10.0984961219092</v>
       </c>
-      <c r="F32" s="15" t="n">
+      <c r="F32" s="11" t="n">
         <f aca="false">EXP(Levers!$G32-Levers!E32)</f>
         <v>8.77666800020352</v>
       </c>
-      <c r="G32" s="15" t="n">
+      <c r="G32" s="11" t="n">
         <f aca="false">EXP(Levers!$G32-Levers!F32)</f>
         <v>10.5402984401513</v>
       </c>
-      <c r="H32" s="15" t="n">
+      <c r="H32" s="11" t="n">
         <f aca="false">B32/C32</f>
         <v>2.7906976744186</v>
       </c>
-      <c r="I32" s="15" t="n">
+      <c r="I32" s="11" t="n">
         <f aca="false">B32/D32</f>
         <v>2.79245283018868</v>
       </c>
-      <c r="J32" s="15" t="n">
+      <c r="J32" s="11" t="n">
         <f aca="false">B32/E32</f>
         <v>1.08421052631579</v>
       </c>
-      <c r="K32" s="15" t="n">
+      <c r="K32" s="11" t="n">
         <f aca="false">B32/F32</f>
         <v>1.24750028086732</v>
       </c>
-      <c r="L32" s="15" t="n">
+      <c r="L32" s="11" t="n">
         <f aca="false">B32/G32</f>
         <v>1.03876525484566</v>
       </c>
-      <c r="M32" s="15"/>
+      <c r="M32" s="11"/>
       <c r="N32" s="9" t="n">
         <f aca="false" t="array" ref="N32:N32">IF(AND(A32&lt;&gt;"gpt-4o-mini",INDEX(Corpus!$Q$3:$Q$60,MATCH(A32,Corpus!$A$3:$A$60,0))&lt;&gt;"None"),1,0)</f>
         <v>1</v>
@@ -8652,55 +8636,55 @@
       </c>
     </row>
     <row r="33" s="1" customFormat="true" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A33" s="15" t="str">
+      <c r="A33" s="11" t="str">
         <f aca="false">Levers!A33</f>
         <v>gpt-5.5 (xhigh)</v>
       </c>
-      <c r="B33" s="15" t="n">
+      <c r="B33" s="11" t="n">
         <f aca="false">Levers!H33</f>
         <v>11.9291597251274</v>
       </c>
-      <c r="C33" s="15" t="n">
+      <c r="C33" s="11" t="n">
         <f aca="false">EXP(Levers!$G33-Levers!B33)</f>
         <v>4.27461556817065</v>
       </c>
-      <c r="D33" s="15" t="n">
+      <c r="D33" s="11" t="n">
         <f aca="false">EXP(Levers!$G33-Levers!C33)</f>
         <v>4.27192882048481</v>
       </c>
-      <c r="E33" s="15" t="n">
+      <c r="E33" s="11" t="n">
         <f aca="false">EXP(Levers!$G33-Levers!D33)</f>
         <v>11.0026230474476</v>
       </c>
-      <c r="F33" s="15" t="n">
+      <c r="F33" s="11" t="n">
         <f aca="false">EXP(Levers!$G33-Levers!E33)</f>
         <v>9.62359634151545</v>
       </c>
-      <c r="G33" s="15" t="n">
+      <c r="G33" s="11" t="n">
         <f aca="false">EXP(Levers!$G33-Levers!F33)</f>
         <v>10.4733281462964</v>
       </c>
-      <c r="H33" s="15" t="n">
+      <c r="H33" s="11" t="n">
         <f aca="false">B33/C33</f>
         <v>2.79069767441861</v>
       </c>
-      <c r="I33" s="15" t="n">
+      <c r="I33" s="11" t="n">
         <f aca="false">B33/D33</f>
         <v>2.79245283018868</v>
       </c>
-      <c r="J33" s="15" t="n">
+      <c r="J33" s="11" t="n">
         <f aca="false">B33/E33</f>
         <v>1.08421052631579</v>
       </c>
-      <c r="K33" s="15" t="n">
+      <c r="K33" s="11" t="n">
         <f aca="false">B33/F33</f>
         <v>1.23957399103139</v>
       </c>
-      <c r="L33" s="15" t="n">
+      <c r="L33" s="11" t="n">
         <f aca="false">B33/G33</f>
         <v>1.13900372054568</v>
       </c>
-      <c r="M33" s="15"/>
+      <c r="M33" s="11"/>
       <c r="N33" s="9" t="n">
         <f aca="false" t="array" ref="N33:N33">IF(AND(A33&lt;&gt;"gpt-4o-mini",INDEX(Corpus!$Q$3:$Q$60,MATCH(A33,Corpus!$A$3:$A$60,0))&lt;&gt;"None"),1,0)</f>
         <v>1</v>
@@ -8723,55 +8707,55 @@
       </c>
     </row>
     <row r="34" s="1" customFormat="true" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A34" s="15" t="str">
+      <c r="A34" s="11" t="str">
         <f aca="false">Levers!A34</f>
         <v>gpt-5.6-luna (minimal)</v>
       </c>
-      <c r="B34" s="15" t="n">
+      <c r="B34" s="11" t="n">
         <f aca="false">Levers!H34</f>
         <v>11.0633144983495</v>
       </c>
-      <c r="C34" s="15" t="n">
+      <c r="C34" s="11" t="n">
         <f aca="false">EXP(Levers!$G34-Levers!B34)</f>
         <v>3.96435436190859</v>
       </c>
-      <c r="D34" s="15" t="n">
+      <c r="D34" s="11" t="n">
         <f aca="false">EXP(Levers!$G34-Levers!C34)</f>
         <v>3.96186262440896</v>
       </c>
-      <c r="E34" s="15" t="n">
+      <c r="E34" s="11" t="n">
         <f aca="false">EXP(Levers!$G34-Levers!D34)</f>
         <v>10.2040279353709</v>
       </c>
-      <c r="F34" s="15" t="n">
+      <c r="F34" s="11" t="n">
         <f aca="false">EXP(Levers!$G34-Levers!E34)</f>
         <v>8.76533500835441</v>
       </c>
-      <c r="G34" s="15" t="n">
+      <c r="G34" s="11" t="n">
         <f aca="false">EXP(Levers!$G34-Levers!F34)</f>
         <v>10.6642175142953</v>
       </c>
-      <c r="H34" s="15" t="n">
+      <c r="H34" s="11" t="n">
         <f aca="false">B34/C34</f>
         <v>2.7906976744186</v>
       </c>
-      <c r="I34" s="15" t="n">
+      <c r="I34" s="11" t="n">
         <f aca="false">B34/D34</f>
         <v>2.79245283018868</v>
       </c>
-      <c r="J34" s="15" t="n">
+      <c r="J34" s="11" t="n">
         <f aca="false">B34/E34</f>
         <v>1.08421052631579</v>
       </c>
-      <c r="K34" s="15" t="n">
+      <c r="K34" s="11" t="n">
         <f aca="false">B34/F34</f>
         <v>1.2621667612025</v>
       </c>
-      <c r="L34" s="15" t="n">
+      <c r="L34" s="11" t="n">
         <f aca="false">B34/G34</f>
         <v>1.03742393509128</v>
       </c>
-      <c r="M34" s="15"/>
+      <c r="M34" s="11"/>
       <c r="N34" s="9" t="n">
         <f aca="false" t="array" ref="N34:N34">IF(AND(A34&lt;&gt;"gpt-4o-mini",INDEX(Corpus!$Q$3:$Q$60,MATCH(A34,Corpus!$A$3:$A$60,0))&lt;&gt;"None"),1,0)</f>
         <v>1</v>
@@ -8794,55 +8778,55 @@
       </c>
     </row>
     <row r="35" s="1" customFormat="true" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A35" s="15" t="str">
+      <c r="A35" s="11" t="str">
         <f aca="false">Levers!A35</f>
         <v>gpt-5.6-luna (low)</v>
       </c>
-      <c r="B35" s="15" t="n">
+      <c r="B35" s="11" t="n">
         <f aca="false">Levers!H35</f>
         <v>10.9006188655751</v>
       </c>
-      <c r="C35" s="15" t="n">
+      <c r="C35" s="11" t="n">
         <f aca="false">EXP(Levers!$G35-Levers!B35)</f>
         <v>3.90605509349774</v>
       </c>
-      <c r="D35" s="15" t="n">
+      <c r="D35" s="11" t="n">
         <f aca="false">EXP(Levers!$G35-Levers!C35)</f>
         <v>3.90359999915865</v>
       </c>
-      <c r="E35" s="15" t="n">
+      <c r="E35" s="11" t="n">
         <f aca="false">EXP(Levers!$G35-Levers!D35)</f>
         <v>10.0539688565984</v>
       </c>
-      <c r="F35" s="15" t="n">
+      <c r="F35" s="11" t="n">
         <f aca="false">EXP(Levers!$G35-Levers!E35)</f>
         <v>8.67168196239032</v>
       </c>
-      <c r="G35" s="15" t="n">
+      <c r="G35" s="11" t="n">
         <f aca="false">EXP(Levers!$G35-Levers!F35)</f>
         <v>10.6208694148178</v>
       </c>
-      <c r="H35" s="15" t="n">
+      <c r="H35" s="11" t="n">
         <f aca="false">B35/C35</f>
         <v>2.79069767441861</v>
       </c>
-      <c r="I35" s="15" t="n">
+      <c r="I35" s="11" t="n">
         <f aca="false">B35/D35</f>
         <v>2.79245283018868</v>
       </c>
-      <c r="J35" s="15" t="n">
+      <c r="J35" s="11" t="n">
         <f aca="false">B35/E35</f>
         <v>1.08421052631579</v>
       </c>
-      <c r="K35" s="15" t="n">
+      <c r="K35" s="11" t="n">
         <f aca="false">B35/F35</f>
         <v>1.25703628348593</v>
       </c>
-      <c r="L35" s="15" t="n">
+      <c r="L35" s="11" t="n">
         <f aca="false">B35/G35</f>
         <v>1.02633959987936</v>
       </c>
-      <c r="M35" s="15"/>
+      <c r="M35" s="11"/>
       <c r="N35" s="9" t="n">
         <f aca="false" t="array" ref="N35:N35">IF(AND(A35&lt;&gt;"gpt-4o-mini",INDEX(Corpus!$Q$3:$Q$60,MATCH(A35,Corpus!$A$3:$A$60,0))&lt;&gt;"None"),1,0)</f>
         <v>1</v>
@@ -8865,55 +8849,55 @@
       </c>
     </row>
     <row r="36" s="1" customFormat="true" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A36" s="15" t="str">
+      <c r="A36" s="11" t="str">
         <f aca="false">Levers!A36</f>
         <v>gpt-5.6-luna (medium)</v>
       </c>
-      <c r="B36" s="15" t="n">
+      <c r="B36" s="11" t="n">
         <f aca="false">Levers!H36</f>
         <v>10.9193489983185</v>
       </c>
-      <c r="C36" s="15" t="n">
+      <c r="C36" s="11" t="n">
         <f aca="false">EXP(Levers!$G36-Levers!B36)</f>
         <v>3.91276672439745</v>
       </c>
-      <c r="D36" s="15" t="n">
+      <c r="D36" s="11" t="n">
         <f aca="false">EXP(Levers!$G36-Levers!C36)</f>
         <v>3.91030741155999</v>
       </c>
-      <c r="E36" s="15" t="n">
+      <c r="E36" s="11" t="n">
         <f aca="false">EXP(Levers!$G36-Levers!D36)</f>
         <v>10.07124422175</v>
       </c>
-      <c r="F36" s="15" t="n">
+      <c r="F36" s="11" t="n">
         <f aca="false">EXP(Levers!$G36-Levers!E36)</f>
         <v>8.68537318076098</v>
       </c>
-      <c r="G36" s="15" t="n">
+      <c r="G36" s="11" t="n">
         <f aca="false">EXP(Levers!$G36-Levers!F36)</f>
         <v>10.6223478521545</v>
       </c>
-      <c r="H36" s="15" t="n">
+      <c r="H36" s="11" t="n">
         <f aca="false">B36/C36</f>
         <v>2.7906976744186</v>
       </c>
-      <c r="I36" s="15" t="n">
+      <c r="I36" s="11" t="n">
         <f aca="false">B36/D36</f>
         <v>2.79245283018868</v>
       </c>
-      <c r="J36" s="15" t="n">
+      <c r="J36" s="11" t="n">
         <f aca="false">B36/E36</f>
         <v>1.08421052631579</v>
       </c>
-      <c r="K36" s="15" t="n">
+      <c r="K36" s="11" t="n">
         <f aca="false">B36/F36</f>
         <v>1.25721126439403</v>
       </c>
-      <c r="L36" s="15" t="n">
+      <c r="L36" s="11" t="n">
         <f aca="false">B36/G36</f>
         <v>1.02796002826284</v>
       </c>
-      <c r="M36" s="15"/>
+      <c r="M36" s="11"/>
       <c r="N36" s="9" t="n">
         <f aca="false" t="array" ref="N36:N36">IF(AND(A36&lt;&gt;"gpt-4o-mini",INDEX(Corpus!$Q$3:$Q$60,MATCH(A36,Corpus!$A$3:$A$60,0))&lt;&gt;"None"),1,0)</f>
         <v>1</v>
@@ -8936,55 +8920,55 @@
       </c>
     </row>
     <row r="37" s="1" customFormat="true" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A37" s="15" t="str">
+      <c r="A37" s="11" t="str">
         <f aca="false">Levers!A37</f>
         <v>gpt-5.6-luna (high)</v>
       </c>
-      <c r="B37" s="15" t="n">
+      <c r="B37" s="11" t="n">
         <f aca="false">Levers!H37</f>
         <v>11.8242991686509</v>
       </c>
-      <c r="C37" s="15" t="n">
+      <c r="C37" s="11" t="n">
         <f aca="false">EXP(Levers!$G37-Levers!B37)</f>
         <v>4.23704053543325</v>
       </c>
-      <c r="D37" s="15" t="n">
+      <c r="D37" s="11" t="n">
         <f aca="false">EXP(Levers!$G37-Levers!C37)</f>
         <v>4.23437740498986</v>
       </c>
-      <c r="E37" s="15" t="n">
+      <c r="E37" s="11" t="n">
         <f aca="false">EXP(Levers!$G37-Levers!D37)</f>
         <v>10.905907000212</v>
       </c>
-      <c r="F37" s="15" t="n">
+      <c r="F37" s="11" t="n">
         <f aca="false">EXP(Levers!$G37-Levers!E37)</f>
         <v>9.42738201799156</v>
       </c>
-      <c r="G37" s="15" t="n">
+      <c r="G37" s="11" t="n">
         <f aca="false">EXP(Levers!$G37-Levers!F37)</f>
         <v>10.5973324546188</v>
       </c>
-      <c r="H37" s="15" t="n">
+      <c r="H37" s="11" t="n">
         <f aca="false">B37/C37</f>
         <v>2.79069767441861</v>
       </c>
-      <c r="I37" s="15" t="n">
+      <c r="I37" s="11" t="n">
         <f aca="false">B37/D37</f>
         <v>2.79245283018868</v>
       </c>
-      <c r="J37" s="15" t="n">
+      <c r="J37" s="11" t="n">
         <f aca="false">B37/E37</f>
         <v>1.08421052631579</v>
       </c>
-      <c r="K37" s="15" t="n">
+      <c r="K37" s="11" t="n">
         <f aca="false">B37/F37</f>
         <v>1.25425055928412</v>
       </c>
-      <c r="L37" s="15" t="n">
+      <c r="L37" s="11" t="n">
         <f aca="false">B37/G37</f>
         <v>1.11578071361698</v>
       </c>
-      <c r="M37" s="15"/>
+      <c r="M37" s="11"/>
       <c r="N37" s="9" t="n">
         <f aca="false" t="array" ref="N37:N37">IF(AND(A37&lt;&gt;"gpt-4o-mini",INDEX(Corpus!$Q$3:$Q$60,MATCH(A37,Corpus!$A$3:$A$60,0))&lt;&gt;"None"),1,0)</f>
         <v>1</v>
@@ -9007,55 +8991,55 @@
       </c>
     </row>
     <row r="38" s="1" customFormat="true" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A38" s="15" t="str">
+      <c r="A38" s="11" t="str">
         <f aca="false">Levers!A38</f>
         <v>gpt-5.6-luna (xhigh)</v>
       </c>
-      <c r="B38" s="15" t="n">
+      <c r="B38" s="11" t="n">
         <f aca="false">Levers!H38</f>
         <v>11.3510697838598</v>
       </c>
-      <c r="C38" s="15" t="n">
+      <c r="C38" s="11" t="n">
         <f aca="false">EXP(Levers!$G38-Levers!B38)</f>
         <v>4.06746667254976</v>
       </c>
-      <c r="D38" s="15" t="n">
+      <c r="D38" s="11" t="n">
         <f aca="false">EXP(Levers!$G38-Levers!C38)</f>
         <v>4.06491012530115</v>
       </c>
-      <c r="E38" s="15" t="n">
+      <c r="E38" s="11" t="n">
         <f aca="false">EXP(Levers!$G38-Levers!D38)</f>
         <v>10.469433295793</v>
       </c>
-      <c r="F38" s="15" t="n">
+      <c r="F38" s="11" t="n">
         <f aca="false">EXP(Levers!$G38-Levers!E38)</f>
         <v>9.04770668524118</v>
       </c>
-      <c r="G38" s="15" t="n">
+      <c r="G38" s="11" t="n">
         <f aca="false">EXP(Levers!$G38-Levers!F38)</f>
         <v>10.6001140113325</v>
       </c>
-      <c r="H38" s="15" t="n">
+      <c r="H38" s="11" t="n">
         <f aca="false">B38/C38</f>
         <v>2.79069767441861</v>
       </c>
-      <c r="I38" s="15" t="n">
+      <c r="I38" s="11" t="n">
         <f aca="false">B38/D38</f>
         <v>2.79245283018868</v>
       </c>
-      <c r="J38" s="15" t="n">
+      <c r="J38" s="11" t="n">
         <f aca="false">B38/E38</f>
         <v>1.08421052631579</v>
       </c>
-      <c r="K38" s="15" t="n">
+      <c r="K38" s="11" t="n">
         <f aca="false">B38/F38</f>
         <v>1.254579771289</v>
       </c>
-      <c r="L38" s="15" t="n">
+      <c r="L38" s="11" t="n">
         <f aca="false">B38/G38</f>
         <v>1.07084412221647</v>
       </c>
-      <c r="M38" s="15"/>
+      <c r="M38" s="11"/>
       <c r="N38" s="9" t="n">
         <f aca="false" t="array" ref="N38:N38">IF(AND(A38&lt;&gt;"gpt-4o-mini",INDEX(Corpus!$Q$3:$Q$60,MATCH(A38,Corpus!$A$3:$A$60,0))&lt;&gt;"None"),1,0)</f>
         <v>1</v>
@@ -9078,55 +9062,55 @@
       </c>
     </row>
     <row r="39" s="1" customFormat="true" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A39" s="15" t="str">
+      <c r="A39" s="11" t="str">
         <f aca="false">Levers!A39</f>
         <v>gpt-5.6-sol (minimal)</v>
       </c>
-      <c r="B39" s="15" t="n">
+      <c r="B39" s="11" t="n">
         <f aca="false">Levers!H39</f>
         <v>10.767984750766</v>
       </c>
-      <c r="C39" s="15" t="n">
+      <c r="C39" s="11" t="n">
         <f aca="false">EXP(Levers!$G39-Levers!B39)</f>
         <v>3.85852786902447</v>
       </c>
-      <c r="D39" s="15" t="n">
+      <c r="D39" s="11" t="n">
         <f aca="false">EXP(Levers!$G39-Levers!C39)</f>
         <v>3.85610264723376</v>
       </c>
-      <c r="E39" s="15" t="n">
+      <c r="E39" s="11" t="n">
         <f aca="false">EXP(Levers!$G39-Levers!D39)</f>
         <v>9.93163642060939</v>
       </c>
-      <c r="F39" s="15" t="n">
+      <c r="F39" s="11" t="n">
         <f aca="false">EXP(Levers!$G39-Levers!E39)</f>
         <v>8.69969033851901</v>
       </c>
-      <c r="G39" s="15" t="n">
+      <c r="G39" s="11" t="n">
         <f aca="false">EXP(Levers!$G39-Levers!F39)</f>
         <v>10.4578616745117</v>
       </c>
-      <c r="H39" s="15" t="n">
+      <c r="H39" s="11" t="n">
         <f aca="false">B39/C39</f>
         <v>2.79069767441861</v>
       </c>
-      <c r="I39" s="15" t="n">
+      <c r="I39" s="11" t="n">
         <f aca="false">B39/D39</f>
         <v>2.79245283018868</v>
       </c>
-      <c r="J39" s="15" t="n">
+      <c r="J39" s="11" t="n">
         <f aca="false">B39/E39</f>
         <v>1.08421052631579</v>
       </c>
-      <c r="K39" s="15" t="n">
+      <c r="K39" s="11" t="n">
         <f aca="false">B39/F39</f>
         <v>1.2377434519812</v>
       </c>
-      <c r="L39" s="15" t="n">
+      <c r="L39" s="11" t="n">
         <f aca="false">B39/G39</f>
         <v>1.02965453989606</v>
       </c>
-      <c r="M39" s="15"/>
+      <c r="M39" s="11"/>
       <c r="N39" s="9" t="n">
         <f aca="false" t="array" ref="N39:N39">IF(AND(A39&lt;&gt;"gpt-4o-mini",INDEX(Corpus!$Q$3:$Q$60,MATCH(A39,Corpus!$A$3:$A$60,0))&lt;&gt;"None"),1,0)</f>
         <v>1</v>
@@ -9149,55 +9133,55 @@
       </c>
     </row>
     <row r="40" s="1" customFormat="true" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A40" s="15" t="str">
+      <c r="A40" s="11" t="str">
         <f aca="false">Levers!A40</f>
         <v>gpt-5.6-sol (low)</v>
       </c>
-      <c r="B40" s="15" t="n">
+      <c r="B40" s="11" t="n">
         <f aca="false">Levers!H40</f>
         <v>10.8631165697576</v>
       </c>
-      <c r="C40" s="15" t="n">
+      <c r="C40" s="11" t="n">
         <f aca="false">EXP(Levers!$G40-Levers!B40)</f>
         <v>3.8926167708298</v>
       </c>
-      <c r="D40" s="15" t="n">
+      <c r="D40" s="11" t="n">
         <f aca="false">EXP(Levers!$G40-Levers!C40)</f>
         <v>3.89017012295373</v>
       </c>
-      <c r="E40" s="15" t="n">
+      <c r="E40" s="11" t="n">
         <f aca="false">EXP(Levers!$G40-Levers!D40)</f>
         <v>10.019379360456</v>
       </c>
-      <c r="F40" s="15" t="n">
+      <c r="F40" s="11" t="n">
         <f aca="false">EXP(Levers!$G40-Levers!E40)</f>
         <v>8.66218167031544</v>
       </c>
-      <c r="G40" s="15" t="n">
+      <c r="G40" s="11" t="n">
         <f aca="false">EXP(Levers!$G40-Levers!F40)</f>
         <v>10.595937981663</v>
       </c>
-      <c r="H40" s="15" t="n">
+      <c r="H40" s="11" t="n">
         <f aca="false">B40/C40</f>
         <v>2.79069767441861</v>
       </c>
-      <c r="I40" s="15" t="n">
+      <c r="I40" s="11" t="n">
         <f aca="false">B40/D40</f>
         <v>2.79245283018868</v>
       </c>
-      <c r="J40" s="15" t="n">
+      <c r="J40" s="11" t="n">
         <f aca="false">B40/E40</f>
         <v>1.08421052631579</v>
       </c>
-      <c r="K40" s="15" t="n">
+      <c r="K40" s="11" t="n">
         <f aca="false">B40/F40</f>
         <v>1.25408551600627</v>
       </c>
-      <c r="L40" s="15" t="n">
+      <c r="L40" s="11" t="n">
         <f aca="false">B40/G40</f>
         <v>1.02521518987342</v>
       </c>
-      <c r="M40" s="15"/>
+      <c r="M40" s="11"/>
       <c r="N40" s="9" t="n">
         <f aca="false" t="array" ref="N40:N40">IF(AND(A40&lt;&gt;"gpt-4o-mini",INDEX(Corpus!$Q$3:$Q$60,MATCH(A40,Corpus!$A$3:$A$60,0))&lt;&gt;"None"),1,0)</f>
         <v>1</v>
@@ -9220,55 +9204,55 @@
       </c>
     </row>
     <row r="41" s="1" customFormat="true" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A41" s="15" t="str">
+      <c r="A41" s="11" t="str">
         <f aca="false">Levers!A41</f>
         <v>gpt-5.6-sol (medium)</v>
       </c>
-      <c r="B41" s="15" t="n">
+      <c r="B41" s="11" t="n">
         <f aca="false">Levers!H41</f>
         <v>10.9368796490469</v>
       </c>
-      <c r="C41" s="15" t="n">
+      <c r="C41" s="11" t="n">
         <f aca="false">EXP(Levers!$G41-Levers!B41)</f>
         <v>3.91904854090846</v>
       </c>
-      <c r="D41" s="15" t="n">
+      <c r="D41" s="11" t="n">
         <f aca="false">EXP(Levers!$G41-Levers!C41)</f>
         <v>3.91658527972624</v>
       </c>
-      <c r="E41" s="15" t="n">
+      <c r="E41" s="11" t="n">
         <f aca="false">EXP(Levers!$G41-Levers!D41)</f>
         <v>10.0874132685384</v>
       </c>
-      <c r="F41" s="15" t="n">
+      <c r="F41" s="11" t="n">
         <f aca="false">EXP(Levers!$G41-Levers!E41)</f>
         <v>8.70451810087942</v>
       </c>
-      <c r="G41" s="15" t="n">
+      <c r="G41" s="11" t="n">
         <f aca="false">EXP(Levers!$G41-Levers!F41)</f>
         <v>10.6160011292635</v>
       </c>
-      <c r="H41" s="15" t="n">
+      <c r="H41" s="11" t="n">
         <f aca="false">B41/C41</f>
         <v>2.7906976744186</v>
       </c>
-      <c r="I41" s="15" t="n">
+      <c r="I41" s="11" t="n">
         <f aca="false">B41/D41</f>
         <v>2.79245283018868</v>
       </c>
-      <c r="J41" s="15" t="n">
+      <c r="J41" s="11" t="n">
         <f aca="false">B41/E41</f>
         <v>1.08421052631579</v>
       </c>
-      <c r="K41" s="15" t="n">
+      <c r="K41" s="11" t="n">
         <f aca="false">B41/F41</f>
         <v>1.25646009604391</v>
       </c>
-      <c r="L41" s="15" t="n">
+      <c r="L41" s="11" t="n">
         <f aca="false">B41/G41</f>
         <v>1.03022593120293</v>
       </c>
-      <c r="M41" s="15"/>
+      <c r="M41" s="11"/>
       <c r="N41" s="9" t="n">
         <f aca="false" t="array" ref="N41:N41">IF(AND(A41&lt;&gt;"gpt-4o-mini",INDEX(Corpus!$Q$3:$Q$60,MATCH(A41,Corpus!$A$3:$A$60,0))&lt;&gt;"None"),1,0)</f>
         <v>1</v>
@@ -9291,55 +9275,55 @@
       </c>
     </row>
     <row r="42" s="1" customFormat="true" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A42" s="15" t="str">
+      <c r="A42" s="11" t="str">
         <f aca="false">Levers!A42</f>
         <v>gpt-5.6-sol (high)</v>
       </c>
-      <c r="B42" s="15" t="n">
+      <c r="B42" s="11" t="n">
         <f aca="false">Levers!H42</f>
         <v>10.8505167559399</v>
       </c>
-      <c r="C42" s="15" t="n">
+      <c r="C42" s="11" t="n">
         <f aca="false">EXP(Levers!$G42-Levers!B42)</f>
         <v>3.88810183754514</v>
       </c>
-      <c r="D42" s="15" t="n">
+      <c r="D42" s="11" t="n">
         <f aca="false">EXP(Levers!$G42-Levers!C42)</f>
         <v>3.88565802746497</v>
       </c>
-      <c r="E42" s="15" t="n">
+      <c r="E42" s="11" t="n">
         <f aca="false">EXP(Levers!$G42-Levers!D42)</f>
         <v>10.0077581729543</v>
       </c>
-      <c r="F42" s="15" t="n">
+      <c r="F42" s="11" t="n">
         <f aca="false">EXP(Levers!$G42-Levers!E42)</f>
         <v>8.66782467491461</v>
       </c>
-      <c r="G42" s="15" t="n">
+      <c r="G42" s="11" t="n">
         <f aca="false">EXP(Levers!$G42-Levers!F42)</f>
         <v>10.5767577994974</v>
       </c>
-      <c r="H42" s="15" t="n">
+      <c r="H42" s="11" t="n">
         <f aca="false">B42/C42</f>
         <v>2.7906976744186</v>
       </c>
-      <c r="I42" s="15" t="n">
+      <c r="I42" s="11" t="n">
         <f aca="false">B42/D42</f>
         <v>2.79245283018868</v>
       </c>
-      <c r="J42" s="15" t="n">
+      <c r="J42" s="11" t="n">
         <f aca="false">B42/E42</f>
         <v>1.08421052631579</v>
       </c>
-      <c r="K42" s="15" t="n">
+      <c r="K42" s="11" t="n">
         <f aca="false">B42/F42</f>
         <v>1.25181543961569</v>
       </c>
-      <c r="L42" s="15" t="n">
+      <c r="L42" s="11" t="n">
         <f aca="false">B42/G42</f>
         <v>1.02588306942753</v>
       </c>
-      <c r="M42" s="15"/>
+      <c r="M42" s="11"/>
       <c r="N42" s="9" t="n">
         <f aca="false" t="array" ref="N42:N42">IF(AND(A42&lt;&gt;"gpt-4o-mini",INDEX(Corpus!$Q$3:$Q$60,MATCH(A42,Corpus!$A$3:$A$60,0))&lt;&gt;"None"),1,0)</f>
         <v>1</v>
@@ -9362,55 +9346,55 @@
       </c>
     </row>
     <row r="43" s="1" customFormat="true" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A43" s="15" t="str">
+      <c r="A43" s="11" t="str">
         <f aca="false">Levers!A43</f>
         <v>gpt-5.6-sol (xhigh)</v>
       </c>
-      <c r="B43" s="15" t="n">
+      <c r="B43" s="11" t="n">
         <f aca="false">Levers!H43</f>
         <v>11.7021359377078</v>
       </c>
-      <c r="C43" s="15" t="n">
+      <c r="C43" s="11" t="n">
         <f aca="false">EXP(Levers!$G43-Levers!B43)</f>
         <v>4.19326537767861</v>
       </c>
-      <c r="D43" s="15" t="n">
+      <c r="D43" s="11" t="n">
         <f aca="false">EXP(Levers!$G43-Levers!C43)</f>
         <v>4.19062976147642</v>
       </c>
-      <c r="E43" s="15" t="n">
+      <c r="E43" s="11" t="n">
         <f aca="false">EXP(Levers!$G43-Levers!D43)</f>
         <v>10.7932321755557</v>
       </c>
-      <c r="F43" s="15" t="n">
+      <c r="F43" s="11" t="n">
         <f aca="false">EXP(Levers!$G43-Levers!E43)</f>
         <v>9.09046859314684</v>
       </c>
-      <c r="G43" s="15" t="n">
+      <c r="G43" s="11" t="n">
         <f aca="false">EXP(Levers!$G43-Levers!F43)</f>
         <v>10.8765490758617</v>
       </c>
-      <c r="H43" s="15" t="n">
+      <c r="H43" s="11" t="n">
         <f aca="false">B43/C43</f>
         <v>2.79069767441861</v>
       </c>
-      <c r="I43" s="15" t="n">
+      <c r="I43" s="11" t="n">
         <f aca="false">B43/D43</f>
         <v>2.79245283018868</v>
       </c>
-      <c r="J43" s="15" t="n">
+      <c r="J43" s="11" t="n">
         <f aca="false">B43/E43</f>
         <v>1.08421052631579</v>
       </c>
-      <c r="K43" s="15" t="n">
+      <c r="K43" s="11" t="n">
         <f aca="false">B43/F43</f>
         <v>1.28729732882305</v>
       </c>
-      <c r="L43" s="15" t="n">
+      <c r="L43" s="11" t="n">
         <f aca="false">B43/G43</f>
         <v>1.07590522104831</v>
       </c>
-      <c r="M43" s="15"/>
+      <c r="M43" s="11"/>
       <c r="N43" s="9" t="n">
         <f aca="false" t="array" ref="N43:N43">IF(AND(A43&lt;&gt;"gpt-4o-mini",INDEX(Corpus!$Q$3:$Q$60,MATCH(A43,Corpus!$A$3:$A$60,0))&lt;&gt;"None"),1,0)</f>
         <v>1</v>
@@ -9433,55 +9417,55 @@
       </c>
     </row>
     <row r="44" s="1" customFormat="true" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A44" s="15" t="str">
+      <c r="A44" s="11" t="str">
         <f aca="false">Levers!A44</f>
         <v>gpt-5.6-sol (max)*</v>
       </c>
-      <c r="B44" s="15" t="n">
+      <c r="B44" s="11" t="n">
         <f aca="false">Levers!H44</f>
         <v>11.7403089074212</v>
       </c>
-      <c r="C44" s="15" t="n">
+      <c r="C44" s="11" t="n">
         <f aca="false">EXP(Levers!$G44-Levers!B44)</f>
         <v>4.20694402515926</v>
       </c>
-      <c r="D44" s="15" t="n">
+      <c r="D44" s="11" t="n">
         <f aca="false">EXP(Levers!$G44-Levers!C44)</f>
         <v>4.20429981144137</v>
       </c>
-      <c r="E44" s="15" t="n">
+      <c r="E44" s="11" t="n">
         <f aca="false">EXP(Levers!$G44-Levers!D44)</f>
         <v>10.8284402544176</v>
       </c>
-      <c r="F44" s="15" t="n">
+      <c r="F44" s="11" t="n">
         <f aca="false">EXP(Levers!$G44-Levers!E44)</f>
         <v>9.09046859314685</v>
       </c>
-      <c r="G44" s="15" t="n">
+      <c r="G44" s="11" t="n">
         <f aca="false">EXP(Levers!$G44-Levers!F44)</f>
         <v>10.9120289387405</v>
       </c>
-      <c r="H44" s="15" t="n">
+      <c r="H44" s="11" t="n">
         <f aca="false">B44/C44</f>
         <v>2.7906976744186</v>
       </c>
-      <c r="I44" s="15" t="n">
+      <c r="I44" s="11" t="n">
         <f aca="false">B44/D44</f>
         <v>2.79245283018868</v>
       </c>
-      <c r="J44" s="15" t="n">
+      <c r="J44" s="11" t="n">
         <f aca="false">B44/E44</f>
         <v>1.08421052631579</v>
       </c>
-      <c r="K44" s="15" t="n">
+      <c r="K44" s="11" t="n">
         <f aca="false">B44/F44</f>
         <v>1.29149655896419</v>
       </c>
-      <c r="L44" s="15" t="n">
+      <c r="L44" s="11" t="n">
         <f aca="false">B44/G44</f>
         <v>1.07590522104831</v>
       </c>
-      <c r="M44" s="15"/>
+      <c r="M44" s="11"/>
       <c r="N44" s="9" t="n">
         <f aca="false" t="array" ref="N44:N44">IF(AND(A44&lt;&gt;"gpt-4o-mini",INDEX(Corpus!$Q$3:$Q$60,MATCH(A44,Corpus!$A$3:$A$60,0))&lt;&gt;"None"),1,0)</f>
         <v>1</v>
@@ -9504,55 +9488,55 @@
       </c>
     </row>
     <row r="45" s="1" customFormat="true" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A45" s="15" t="str">
+      <c r="A45" s="11" t="str">
         <f aca="false">Levers!A45</f>
         <v>gpt-5.6-terra (minimal)</v>
       </c>
-      <c r="B45" s="15" t="n">
+      <c r="B45" s="11" t="n">
         <f aca="false">Levers!H45</f>
         <v>11.0476220354167</v>
       </c>
-      <c r="C45" s="15" t="n">
+      <c r="C45" s="11" t="n">
         <f aca="false">EXP(Levers!$G45-Levers!B45)</f>
         <v>3.95873122935764</v>
       </c>
-      <c r="D45" s="15" t="n">
+      <c r="D45" s="11" t="n">
         <f aca="false">EXP(Levers!$G45-Levers!C45)</f>
         <v>3.95624302619651</v>
       </c>
-      <c r="E45" s="15" t="n">
+      <c r="E45" s="11" t="n">
         <f aca="false">EXP(Levers!$G45-Levers!D45)</f>
         <v>10.1895543045105</v>
       </c>
-      <c r="F45" s="15" t="n">
+      <c r="F45" s="11" t="n">
         <f aca="false">EXP(Levers!$G45-Levers!E45)</f>
         <v>8.81021657039537</v>
       </c>
-      <c r="G45" s="15" t="n">
+      <c r="G45" s="11" t="n">
         <f aca="false">EXP(Levers!$G45-Levers!F45)</f>
         <v>10.5948418667333</v>
       </c>
-      <c r="H45" s="15" t="n">
+      <c r="H45" s="11" t="n">
         <f aca="false">B45/C45</f>
         <v>2.7906976744186</v>
       </c>
-      <c r="I45" s="15" t="n">
+      <c r="I45" s="11" t="n">
         <f aca="false">B45/D45</f>
         <v>2.79245283018868</v>
       </c>
-      <c r="J45" s="15" t="n">
+      <c r="J45" s="11" t="n">
         <f aca="false">B45/E45</f>
         <v>1.08421052631579</v>
       </c>
-      <c r="K45" s="15" t="n">
+      <c r="K45" s="11" t="n">
         <f aca="false">B45/F45</f>
         <v>1.25395578498485</v>
       </c>
-      <c r="L45" s="15" t="n">
+      <c r="L45" s="11" t="n">
         <f aca="false">B45/G45</f>
         <v>1.04273590624369</v>
       </c>
-      <c r="M45" s="15"/>
+      <c r="M45" s="11"/>
       <c r="N45" s="9" t="n">
         <f aca="false" t="array" ref="N45:N45">IF(AND(A45&lt;&gt;"gpt-4o-mini",INDEX(Corpus!$Q$3:$Q$60,MATCH(A45,Corpus!$A$3:$A$60,0))&lt;&gt;"None"),1,0)</f>
         <v>1</v>
@@ -9575,55 +9559,55 @@
       </c>
     </row>
     <row r="46" s="1" customFormat="true" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A46" s="15" t="str">
+      <c r="A46" s="11" t="str">
         <f aca="false">Levers!A46</f>
         <v>gpt-5.6-terra (low)</v>
       </c>
-      <c r="B46" s="15" t="n">
+      <c r="B46" s="11" t="n">
         <f aca="false">Levers!H46</f>
         <v>10.641683080279</v>
       </c>
-      <c r="C46" s="15" t="n">
+      <c r="C46" s="11" t="n">
         <f aca="false">EXP(Levers!$G46-Levers!B46)</f>
         <v>3.8132697704333</v>
       </c>
-      <c r="D46" s="15" t="n">
+      <c r="D46" s="11" t="n">
         <f aca="false">EXP(Levers!$G46-Levers!C46)</f>
         <v>3.81087299496477</v>
       </c>
-      <c r="E46" s="15" t="n">
+      <c r="E46" s="11" t="n">
         <f aca="false">EXP(Levers!$G46-Levers!D46)</f>
         <v>9.81514458860682</v>
       </c>
-      <c r="F46" s="15" t="n">
+      <c r="F46" s="11" t="n">
         <f aca="false">EXP(Levers!$G46-Levers!E46)</f>
         <v>8.67496058503691</v>
       </c>
-      <c r="G46" s="15" t="n">
+      <c r="G46" s="11" t="n">
         <f aca="false">EXP(Levers!$G46-Levers!F46)</f>
         <v>10.3646601514347</v>
       </c>
-      <c r="H46" s="15" t="n">
+      <c r="H46" s="11" t="n">
         <f aca="false">B46/C46</f>
         <v>2.7906976744186</v>
       </c>
-      <c r="I46" s="15" t="n">
+      <c r="I46" s="11" t="n">
         <f aca="false">B46/D46</f>
         <v>2.79245283018868</v>
       </c>
-      <c r="J46" s="15" t="n">
+      <c r="J46" s="11" t="n">
         <f aca="false">B46/E46</f>
         <v>1.08421052631579</v>
       </c>
-      <c r="K46" s="15" t="n">
+      <c r="K46" s="11" t="n">
         <f aca="false">B46/F46</f>
         <v>1.22671255690019</v>
       </c>
-      <c r="L46" s="15" t="n">
+      <c r="L46" s="11" t="n">
         <f aca="false">B46/G46</f>
         <v>1.02672764227642</v>
       </c>
-      <c r="M46" s="15"/>
+      <c r="M46" s="11"/>
       <c r="N46" s="9" t="n">
         <f aca="false" t="array" ref="N46:N46">IF(AND(A46&lt;&gt;"gpt-4o-mini",INDEX(Corpus!$Q$3:$Q$60,MATCH(A46,Corpus!$A$3:$A$60,0))&lt;&gt;"None"),1,0)</f>
         <v>1</v>
@@ -9646,55 +9630,55 @@
       </c>
     </row>
     <row r="47" s="1" customFormat="true" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A47" s="15" t="str">
+      <c r="A47" s="11" t="str">
         <f aca="false">Levers!A47</f>
         <v>gpt-5.6-terra (medium)</v>
       </c>
-      <c r="B47" s="15" t="n">
+      <c r="B47" s="11" t="n">
         <f aca="false">Levers!H47</f>
         <v>10.6800966228628</v>
       </c>
-      <c r="C47" s="15" t="n">
+      <c r="C47" s="11" t="n">
         <f aca="false">EXP(Levers!$G47-Levers!B47)</f>
         <v>3.82703462319251</v>
       </c>
-      <c r="D47" s="15" t="n">
+      <c r="D47" s="11" t="n">
         <f aca="false">EXP(Levers!$G47-Levers!C47)</f>
         <v>3.8246291960252</v>
       </c>
-      <c r="E47" s="15" t="n">
+      <c r="E47" s="11" t="n">
         <f aca="false">EXP(Levers!$G47-Levers!D47)</f>
         <v>9.85057455506765</v>
       </c>
-      <c r="F47" s="15" t="n">
+      <c r="F47" s="11" t="n">
         <f aca="false">EXP(Levers!$G47-Levers!E47)</f>
         <v>8.69105554063296</v>
       </c>
-      <c r="G47" s="15" t="n">
+      <c r="G47" s="11" t="n">
         <f aca="false">EXP(Levers!$G47-Levers!F47)</f>
         <v>10.3828101294478</v>
       </c>
-      <c r="H47" s="15" t="n">
+      <c r="H47" s="11" t="n">
         <f aca="false">B47/C47</f>
         <v>2.79069767441861</v>
       </c>
-      <c r="I47" s="15" t="n">
+      <c r="I47" s="11" t="n">
         <f aca="false">B47/D47</f>
         <v>2.79245283018868</v>
       </c>
-      <c r="J47" s="15" t="n">
+      <c r="J47" s="11" t="n">
         <f aca="false">B47/E47</f>
         <v>1.08421052631579</v>
       </c>
-      <c r="K47" s="15" t="n">
+      <c r="K47" s="11" t="n">
         <f aca="false">B47/F47</f>
         <v>1.22886070315977</v>
       </c>
-      <c r="L47" s="15" t="n">
+      <c r="L47" s="11" t="n">
         <f aca="false">B47/G47</f>
         <v>1.02863256572244</v>
       </c>
-      <c r="M47" s="15"/>
+      <c r="M47" s="11"/>
       <c r="N47" s="9" t="n">
         <f aca="false" t="array" ref="N47:N47">IF(AND(A47&lt;&gt;"gpt-4o-mini",INDEX(Corpus!$Q$3:$Q$60,MATCH(A47,Corpus!$A$3:$A$60,0))&lt;&gt;"None"),1,0)</f>
         <v>1</v>
@@ -9717,55 +9701,55 @@
       </c>
     </row>
     <row r="48" s="1" customFormat="true" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A48" s="15" t="str">
+      <c r="A48" s="11" t="str">
         <f aca="false">Levers!A48</f>
         <v>gpt-5.6-terra (high)</v>
       </c>
-      <c r="B48" s="15" t="n">
+      <c r="B48" s="11" t="n">
         <f aca="false">Levers!H48</f>
         <v>10.7829327969148</v>
       </c>
-      <c r="C48" s="15" t="n">
+      <c r="C48" s="11" t="n">
         <f aca="false">EXP(Levers!$G48-Levers!B48)</f>
         <v>3.8638842522278</v>
       </c>
-      <c r="D48" s="15" t="n">
+      <c r="D48" s="11" t="n">
         <f aca="false">EXP(Levers!$G48-Levers!C48)</f>
         <v>3.86145566376002</v>
       </c>
-      <c r="E48" s="15" t="n">
+      <c r="E48" s="11" t="n">
         <f aca="false">EXP(Levers!$G48-Levers!D48)</f>
         <v>9.94542345346509</v>
       </c>
-      <c r="F48" s="15" t="n">
+      <c r="F48" s="11" t="n">
         <f aca="false">EXP(Levers!$G48-Levers!E48)</f>
         <v>8.61009536363576</v>
       </c>
-      <c r="G48" s="15" t="n">
+      <c r="G48" s="11" t="n">
         <f aca="false">EXP(Levers!$G48-Levers!F48)</f>
         <v>10.5813527475956</v>
       </c>
-      <c r="H48" s="15" t="n">
+      <c r="H48" s="11" t="n">
         <f aca="false">B48/C48</f>
         <v>2.7906976744186</v>
       </c>
-      <c r="I48" s="15" t="n">
+      <c r="I48" s="11" t="n">
         <f aca="false">B48/D48</f>
         <v>2.79245283018868</v>
       </c>
-      <c r="J48" s="15" t="n">
+      <c r="J48" s="11" t="n">
         <f aca="false">B48/E48</f>
         <v>1.08421052631579</v>
       </c>
-      <c r="K48" s="15" t="n">
+      <c r="K48" s="11" t="n">
         <f aca="false">B48/F48</f>
         <v>1.25235927611857</v>
       </c>
-      <c r="L48" s="15" t="n">
+      <c r="L48" s="11" t="n">
         <f aca="false">B48/G48</f>
         <v>1.01905049894164</v>
       </c>
-      <c r="M48" s="15"/>
+      <c r="M48" s="11"/>
       <c r="N48" s="9" t="n">
         <f aca="false" t="array" ref="N48:N48">IF(AND(A48&lt;&gt;"gpt-4o-mini",INDEX(Corpus!$Q$3:$Q$60,MATCH(A48,Corpus!$A$3:$A$60,0))&lt;&gt;"None"),1,0)</f>
         <v>1</v>
@@ -9788,55 +9772,55 @@
       </c>
     </row>
     <row r="49" s="1" customFormat="true" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A49" s="15" t="str">
+      <c r="A49" s="11" t="str">
         <f aca="false">Levers!A49</f>
         <v>gpt-5.6-terra (xhigh)</v>
       </c>
-      <c r="B49" s="15" t="n">
+      <c r="B49" s="11" t="n">
         <f aca="false">Levers!H49</f>
         <v>11.0109892265593</v>
       </c>
-      <c r="C49" s="15" t="n">
+      <c r="C49" s="11" t="n">
         <f aca="false">EXP(Levers!$G49-Levers!B49)</f>
         <v>3.94560447285041</v>
       </c>
-      <c r="D49" s="15" t="n">
+      <c r="D49" s="11" t="n">
         <f aca="false">EXP(Levers!$G49-Levers!C49)</f>
         <v>3.9431245203219</v>
       </c>
-      <c r="E49" s="15" t="n">
+      <c r="E49" s="11" t="n">
         <f aca="false">EXP(Levers!$G49-Levers!D49)</f>
         <v>10.1557667623605</v>
       </c>
-      <c r="F49" s="15" t="n">
+      <c r="F49" s="11" t="n">
         <f aca="false">EXP(Levers!$G49-Levers!E49)</f>
         <v>8.86786406550118</v>
       </c>
-      <c r="G49" s="15" t="n">
+      <c r="G49" s="11" t="n">
         <f aca="false">EXP(Levers!$G49-Levers!F49)</f>
         <v>10.4910647181588</v>
       </c>
-      <c r="H49" s="15" t="n">
+      <c r="H49" s="11" t="n">
         <f aca="false">B49/C49</f>
         <v>2.7906976744186</v>
       </c>
-      <c r="I49" s="15" t="n">
+      <c r="I49" s="11" t="n">
         <f aca="false">B49/D49</f>
         <v>2.79245283018868</v>
       </c>
-      <c r="J49" s="15" t="n">
+      <c r="J49" s="11" t="n">
         <f aca="false">B49/E49</f>
         <v>1.08421052631579</v>
       </c>
-      <c r="K49" s="15" t="n">
+      <c r="K49" s="11" t="n">
         <f aca="false">B49/F49</f>
         <v>1.24167320847819</v>
       </c>
-      <c r="L49" s="15" t="n">
+      <c r="L49" s="11" t="n">
         <f aca="false">B49/G49</f>
         <v>1.04955879335112</v>
       </c>
-      <c r="M49" s="15"/>
+      <c r="M49" s="11"/>
       <c r="N49" s="9" t="n">
         <f aca="false" t="array" ref="N49:N49">IF(AND(A49&lt;&gt;"gpt-4o-mini",INDEX(Corpus!$Q$3:$Q$60,MATCH(A49,Corpus!$A$3:$A$60,0))&lt;&gt;"None"),1,0)</f>
         <v>1</v>
@@ -9859,162 +9843,162 @@
       </c>
     </row>
     <row r="50" s="1" customFormat="true" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A50" s="15"/>
-      <c r="B50" s="15"/>
-      <c r="C50" s="15"/>
-      <c r="D50" s="15"/>
-      <c r="E50" s="15"/>
-      <c r="F50" s="15"/>
-      <c r="G50" s="15"/>
-      <c r="H50" s="15"/>
-      <c r="I50" s="15"/>
-      <c r="J50" s="15"/>
-      <c r="K50" s="15"/>
-      <c r="L50" s="15"/>
-      <c r="M50" s="15"/>
+      <c r="A50" s="11"/>
+      <c r="B50" s="11"/>
+      <c r="C50" s="11"/>
+      <c r="D50" s="11"/>
+      <c r="E50" s="11"/>
+      <c r="F50" s="11"/>
+      <c r="G50" s="11"/>
+      <c r="H50" s="11"/>
+      <c r="I50" s="11"/>
+      <c r="J50" s="11"/>
+      <c r="K50" s="11"/>
+      <c r="L50" s="11"/>
+      <c r="M50" s="11"/>
     </row>
     <row r="51" s="1" customFormat="true" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A51" s="15" t="s">
+      <c r="A51" s="11" t="s">
         <v>279</v>
       </c>
-      <c r="B51" s="15" t="n">
+      <c r="B51" s="11" t="n">
         <f aca="false" t="array" ref="B51:B51">MEDIAN(IF($N$3:$N$49=1,B3:B49))</f>
         <v>11.0843005102309</v>
       </c>
-      <c r="C51" s="15" t="n">
+      <c r="C51" s="11" t="n">
         <f aca="false" t="array" ref="C51:C51">MEDIAN(IF($N$3:$N$49=1,C3:C49))</f>
         <v>3.97187434949939</v>
       </c>
-      <c r="D51" s="15" t="n">
+      <c r="D51" s="11" t="n">
         <f aca="false" t="array" ref="D51:D51">MEDIAN(IF($N$3:$N$49=1,D3:D49))</f>
         <v>3.96937788542051</v>
       </c>
-      <c r="E51" s="15" t="n">
+      <c r="E51" s="11" t="n">
         <f aca="false" t="array" ref="E51:E51">MEDIAN(IF($N$3:$N$49=1,E3:E49))</f>
         <v>10.2233839657469</v>
       </c>
-      <c r="F51" s="15" t="n">
+      <c r="F51" s="11" t="n">
         <f aca="false" t="array" ref="F51:F51">MEDIAN(IF($N$3:$N$49=1,F3:F49))</f>
         <v>8.91483548505999</v>
       </c>
-      <c r="G51" s="15" t="n">
+      <c r="G51" s="11" t="n">
         <f aca="false" t="array" ref="G51:G51">MEDIAN(IF($N$3:$N$49=1,G3:G49))</f>
         <v>10.5767577994974</v>
       </c>
-      <c r="H51" s="15" t="n">
+      <c r="H51" s="11" t="n">
         <f aca="false" t="array" ref="H51:H51">MEDIAN(IF($N$3:$N$49=1,H3:H49))</f>
         <v>2.7906976744186</v>
       </c>
-      <c r="I51" s="15" t="n">
+      <c r="I51" s="11" t="n">
         <f aca="false" t="array" ref="I51:I51">MEDIAN(IF($N$3:$N$49=1,I3:I49))</f>
         <v>2.79245283018868</v>
       </c>
-      <c r="J51" s="15" t="n">
+      <c r="J51" s="11" t="n">
         <f aca="false" t="array" ref="J51:J51">MEDIAN(IF($N$3:$N$49=1,J3:J49))</f>
         <v>1.08421052631579</v>
       </c>
-      <c r="K51" s="15" t="n">
+      <c r="K51" s="11" t="n">
         <f aca="false" t="array" ref="K51:K51">MEDIAN(IF($N$3:$N$49=1,K3:K49))</f>
         <v>1.25181543961569</v>
       </c>
-      <c r="L51" s="15" t="n">
+      <c r="L51" s="11" t="n">
         <f aca="false" t="array" ref="L51:L51">MEDIAN(IF($N$3:$N$49=1,L3:L49))</f>
         <v>1.05511811023622</v>
       </c>
-      <c r="M51" s="15"/>
+      <c r="M51" s="11"/>
     </row>
     <row r="52" s="1" customFormat="true" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A52" s="15" t="s">
+      <c r="A52" s="11" t="s">
         <v>280</v>
       </c>
-      <c r="B52" s="15" t="n">
+      <c r="B52" s="11" t="n">
         <f aca="false" t="array" ref="B52:B52">MEDIAN(IF($N$3:$N$49=1,$O$3:$O$49))</f>
         <v>1.42236040894235</v>
       </c>
-      <c r="C52" s="15" t="n">
+      <c r="C52" s="11" t="n">
         <f aca="false" t="array" ref="C52:C52">MIN(IF($N$3:$N$49=1,$O$3:$O$49))</f>
         <v>1.36556282319571</v>
       </c>
-      <c r="D52" s="15" t="n">
+      <c r="D52" s="11" t="n">
         <f aca="false" t="array" ref="D52:D52">MAX(IF($N$3:$N$49=1,$O$3:$O$49))</f>
         <v>2.42524805705106</v>
       </c>
-      <c r="E52" s="15"/>
-      <c r="F52" s="15"/>
-      <c r="G52" s="15"/>
-      <c r="H52" s="15"/>
-      <c r="I52" s="15"/>
-      <c r="J52" s="15"/>
-      <c r="K52" s="15"/>
-      <c r="L52" s="15"/>
-      <c r="M52" s="15"/>
+      <c r="E52" s="11"/>
+      <c r="F52" s="11"/>
+      <c r="G52" s="11"/>
+      <c r="H52" s="11"/>
+      <c r="I52" s="11"/>
+      <c r="J52" s="11"/>
+      <c r="K52" s="11"/>
+      <c r="L52" s="11"/>
+      <c r="M52" s="11"/>
     </row>
     <row r="53" s="1" customFormat="true" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A53" s="15" t="s">
+      <c r="A53" s="11" t="s">
         <v>281</v>
       </c>
-      <c r="B53" s="15" t="n">
+      <c r="B53" s="11" t="n">
         <f aca="false" t="array" ref="B53:B53">MIN(IF($N$3:$N$49=1,$B$3:$B$49))</f>
         <v>10.641683080279</v>
       </c>
-      <c r="C53" s="15" t="n">
+      <c r="C53" s="11" t="n">
         <f aca="false" t="array" ref="C53:C53">MEDIAN(IF($N$3:$N$49=1,$B$3:$B$49))</f>
         <v>11.0843005102309</v>
       </c>
-      <c r="D53" s="15" t="n">
+      <c r="D53" s="11" t="n">
         <f aca="false" t="array" ref="D53:D53">AVERAGE(IF($N$3:$N$49=1,$B$3:$B$49))</f>
         <v>11.4797470751577</v>
       </c>
-      <c r="E53" s="15" t="n">
+      <c r="E53" s="11" t="n">
         <f aca="false" t="array" ref="E53:E53">MAX(IF($N$3:$N$49=1,$B$3:$B$49))</f>
         <v>18.8996952581074</v>
       </c>
-      <c r="F53" s="15"/>
-      <c r="G53" s="15"/>
-      <c r="H53" s="15"/>
-      <c r="I53" s="15"/>
-      <c r="J53" s="15"/>
-      <c r="K53" s="15"/>
-      <c r="L53" s="15"/>
-      <c r="M53" s="15"/>
+      <c r="F53" s="11"/>
+      <c r="G53" s="11"/>
+      <c r="H53" s="11"/>
+      <c r="I53" s="11"/>
+      <c r="J53" s="11"/>
+      <c r="K53" s="11"/>
+      <c r="L53" s="11"/>
+      <c r="M53" s="11"/>
     </row>
     <row r="54" s="1" customFormat="true" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A54" s="15" t="s">
+      <c r="A54" s="11" t="s">
         <v>282</v>
       </c>
-      <c r="B54" s="15" t="n">
+      <c r="B54" s="11" t="n">
         <f aca="false" t="array" ref="B54:B54">MEDIAN(IF($N$3:$N$49=1,$P$3:$P$49))</f>
         <v>1.14397016162453</v>
       </c>
-      <c r="C54" s="15" t="n">
+      <c r="C54" s="11" t="n">
         <f aca="false" t="array" ref="C54:C54">MEDIAN(IF($N$3:$N$49=1,$Q$3:$Q$49))</f>
         <v>1.08421052631579</v>
       </c>
-      <c r="D54" s="15" t="n">
+      <c r="D54" s="11" t="n">
         <f aca="false" t="array" ref="D54:D54">MEDIAN(IF($N$3:$N$49=1,$R$3:$R$49))</f>
         <v>1</v>
       </c>
-      <c r="E54" s="15" t="n">
+      <c r="E54" s="11" t="n">
         <f aca="false">$B$51/B54</f>
         <v>9.68932659440192</v>
       </c>
-      <c r="F54" s="15" t="n">
+      <c r="F54" s="11" t="n">
         <f aca="false">$B$51/C54</f>
         <v>10.2233839657469</v>
       </c>
-      <c r="G54" s="15" t="n">
+      <c r="G54" s="11" t="n">
         <f aca="false">$B$51/D54</f>
         <v>11.0843005102309</v>
       </c>
-      <c r="H54" s="15" t="n">
+      <c r="H54" s="11" t="n">
         <f aca="false">$B$51/$B$52</f>
         <v>7.7928916191312</v>
       </c>
-      <c r="I54" s="15"/>
-      <c r="J54" s="15"/>
-      <c r="K54" s="15"/>
-      <c r="L54" s="15"/>
-      <c r="M54" s="15"/>
+      <c r="I54" s="11"/>
+      <c r="J54" s="11"/>
+      <c r="K54" s="11"/>
+      <c r="L54" s="11"/>
+      <c r="M54" s="11"/>
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
@@ -10039,92 +10023,92 @@
   </cols>
   <sheetData>
     <row r="1" s="1" customFormat="true" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1" s="17" t="s">
+      <c r="A1" s="13" t="s">
         <v>283</v>
       </c>
-      <c r="B1" s="17"/>
-      <c r="C1" s="17"/>
-      <c r="D1" s="17"/>
-      <c r="E1" s="17"/>
-      <c r="F1" s="17"/>
-      <c r="G1" s="17"/>
-      <c r="H1" s="17"/>
-      <c r="I1" s="17"/>
-      <c r="J1" s="17"/>
-      <c r="K1" s="17"/>
-      <c r="L1" s="17"/>
-      <c r="M1" s="17"/>
-      <c r="N1" s="17"/>
-      <c r="O1" s="17"/>
-      <c r="P1" s="17"/>
-      <c r="Q1" s="17"/>
-      <c r="R1" s="17"/>
-      <c r="S1" s="17"/>
-      <c r="T1" s="17"/>
-      <c r="U1" s="17"/>
+      <c r="B1" s="13"/>
+      <c r="C1" s="13"/>
+      <c r="D1" s="13"/>
+      <c r="E1" s="13"/>
+      <c r="F1" s="13"/>
+      <c r="G1" s="13"/>
+      <c r="H1" s="13"/>
+      <c r="I1" s="13"/>
+      <c r="J1" s="13"/>
+      <c r="K1" s="13"/>
+      <c r="L1" s="13"/>
+      <c r="M1" s="13"/>
+      <c r="N1" s="13"/>
+      <c r="O1" s="13"/>
+      <c r="P1" s="13"/>
+      <c r="Q1" s="13"/>
+      <c r="R1" s="13"/>
+      <c r="S1" s="13"/>
+      <c r="T1" s="13"/>
+      <c r="U1" s="13"/>
     </row>
     <row r="2" s="1" customFormat="true" ht="69.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A2" s="18" t="s">
+      <c r="A2" s="14" t="s">
         <v>284</v>
       </c>
-      <c r="B2" s="18" t="s">
+      <c r="B2" s="14" t="s">
         <v>285</v>
       </c>
-      <c r="C2" s="18" t="s">
+      <c r="C2" s="14" t="s">
         <v>286</v>
       </c>
-      <c r="D2" s="18" t="s">
+      <c r="D2" s="14" t="s">
         <v>287</v>
       </c>
-      <c r="E2" s="18" t="s">
+      <c r="E2" s="14" t="s">
         <v>288</v>
       </c>
-      <c r="F2" s="18" t="s">
+      <c r="F2" s="14" t="s">
         <v>289</v>
       </c>
-      <c r="G2" s="18" t="s">
+      <c r="G2" s="14" t="s">
         <v>290</v>
       </c>
-      <c r="H2" s="18" t="s">
+      <c r="H2" s="14" t="s">
         <v>291</v>
       </c>
-      <c r="I2" s="18" t="s">
+      <c r="I2" s="14" t="s">
         <v>292</v>
       </c>
-      <c r="J2" s="18" t="s">
+      <c r="J2" s="14" t="s">
         <v>293</v>
       </c>
-      <c r="K2" s="18" t="s">
+      <c r="K2" s="14" t="s">
         <v>294</v>
       </c>
-      <c r="L2" s="18" t="s">
+      <c r="L2" s="14" t="s">
         <v>295</v>
       </c>
-      <c r="M2" s="18" t="s">
+      <c r="M2" s="14" t="s">
         <v>296</v>
       </c>
-      <c r="N2" s="18" t="s">
+      <c r="N2" s="14" t="s">
         <v>297</v>
       </c>
-      <c r="O2" s="18" t="s">
+      <c r="O2" s="14" t="s">
         <v>298</v>
       </c>
-      <c r="P2" s="18" t="s">
+      <c r="P2" s="14" t="s">
         <v>299</v>
       </c>
-      <c r="Q2" s="18" t="s">
+      <c r="Q2" s="14" t="s">
         <v>300</v>
       </c>
-      <c r="R2" s="18" t="s">
+      <c r="R2" s="14" t="s">
         <v>301</v>
       </c>
-      <c r="S2" s="18" t="s">
+      <c r="S2" s="14" t="s">
         <v>302</v>
       </c>
-      <c r="T2" s="18" t="s">
+      <c r="T2" s="14" t="s">
         <v>303</v>
       </c>
-      <c r="U2" s="18" t="s">
+      <c r="U2" s="14" t="s">
         <v>304</v>
       </c>
     </row>
@@ -11019,190 +11003,190 @@
       <c r="A17" s="2" t="s">
         <v>308</v>
       </c>
-      <c r="B17" s="17" t="s">
+      <c r="B17" s="13" t="s">
         <v>309</v>
       </c>
-      <c r="C17" s="17"/>
-      <c r="D17" s="17"/>
-      <c r="E17" s="17"/>
-      <c r="F17" s="17"/>
-      <c r="G17" s="17"/>
-      <c r="H17" s="17"/>
-      <c r="I17" s="17"/>
-      <c r="J17" s="17"/>
-      <c r="K17" s="17"/>
-      <c r="L17" s="17"/>
-      <c r="M17" s="17"/>
-      <c r="N17" s="17"/>
-      <c r="O17" s="17"/>
-      <c r="P17" s="17"/>
-      <c r="Q17" s="17"/>
-      <c r="R17" s="17"/>
-      <c r="S17" s="17"/>
-      <c r="T17" s="17"/>
-      <c r="U17" s="17"/>
+      <c r="C17" s="13"/>
+      <c r="D17" s="13"/>
+      <c r="E17" s="13"/>
+      <c r="F17" s="13"/>
+      <c r="G17" s="13"/>
+      <c r="H17" s="13"/>
+      <c r="I17" s="13"/>
+      <c r="J17" s="13"/>
+      <c r="K17" s="13"/>
+      <c r="L17" s="13"/>
+      <c r="M17" s="13"/>
+      <c r="N17" s="13"/>
+      <c r="O17" s="13"/>
+      <c r="P17" s="13"/>
+      <c r="Q17" s="13"/>
+      <c r="R17" s="13"/>
+      <c r="S17" s="13"/>
+      <c r="T17" s="13"/>
+      <c r="U17" s="13"/>
     </row>
     <row r="18" s="1" customFormat="true" ht="57.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="2" t="s">
         <v>310</v>
       </c>
-      <c r="B18" s="17" t="s">
+      <c r="B18" s="13" t="s">
         <v>311</v>
       </c>
-      <c r="C18" s="17"/>
-      <c r="D18" s="17"/>
-      <c r="E18" s="17"/>
-      <c r="F18" s="17"/>
-      <c r="G18" s="17"/>
-      <c r="H18" s="17"/>
-      <c r="I18" s="17"/>
-      <c r="J18" s="17"/>
-      <c r="K18" s="17"/>
-      <c r="L18" s="17"/>
-      <c r="M18" s="17"/>
-      <c r="N18" s="17"/>
-      <c r="O18" s="17"/>
-      <c r="P18" s="17"/>
-      <c r="Q18" s="17"/>
-      <c r="R18" s="17"/>
-      <c r="S18" s="17"/>
-      <c r="T18" s="17"/>
-      <c r="U18" s="17"/>
+      <c r="C18" s="13"/>
+      <c r="D18" s="13"/>
+      <c r="E18" s="13"/>
+      <c r="F18" s="13"/>
+      <c r="G18" s="13"/>
+      <c r="H18" s="13"/>
+      <c r="I18" s="13"/>
+      <c r="J18" s="13"/>
+      <c r="K18" s="13"/>
+      <c r="L18" s="13"/>
+      <c r="M18" s="13"/>
+      <c r="N18" s="13"/>
+      <c r="O18" s="13"/>
+      <c r="P18" s="13"/>
+      <c r="Q18" s="13"/>
+      <c r="R18" s="13"/>
+      <c r="S18" s="13"/>
+      <c r="T18" s="13"/>
+      <c r="U18" s="13"/>
     </row>
     <row r="19" s="1" customFormat="true" ht="57.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="2" t="s">
         <v>312</v>
       </c>
-      <c r="B19" s="17" t="s">
+      <c r="B19" s="13" t="s">
         <v>313</v>
       </c>
-      <c r="C19" s="17"/>
-      <c r="D19" s="17"/>
-      <c r="E19" s="17"/>
-      <c r="F19" s="17"/>
-      <c r="G19" s="17"/>
-      <c r="H19" s="17"/>
-      <c r="I19" s="17"/>
-      <c r="J19" s="17"/>
-      <c r="K19" s="17"/>
-      <c r="L19" s="17"/>
-      <c r="M19" s="17"/>
-      <c r="N19" s="17"/>
-      <c r="O19" s="17"/>
-      <c r="P19" s="17"/>
-      <c r="Q19" s="17"/>
-      <c r="R19" s="17"/>
-      <c r="S19" s="17"/>
-      <c r="T19" s="17"/>
-      <c r="U19" s="17"/>
+      <c r="C19" s="13"/>
+      <c r="D19" s="13"/>
+      <c r="E19" s="13"/>
+      <c r="F19" s="13"/>
+      <c r="G19" s="13"/>
+      <c r="H19" s="13"/>
+      <c r="I19" s="13"/>
+      <c r="J19" s="13"/>
+      <c r="K19" s="13"/>
+      <c r="L19" s="13"/>
+      <c r="M19" s="13"/>
+      <c r="N19" s="13"/>
+      <c r="O19" s="13"/>
+      <c r="P19" s="13"/>
+      <c r="Q19" s="13"/>
+      <c r="R19" s="13"/>
+      <c r="S19" s="13"/>
+      <c r="T19" s="13"/>
+      <c r="U19" s="13"/>
     </row>
     <row r="20" s="1" customFormat="true" ht="57.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="2" t="s">
         <v>314</v>
       </c>
-      <c r="B20" s="17" t="s">
+      <c r="B20" s="13" t="s">
         <v>315</v>
       </c>
-      <c r="C20" s="17"/>
-      <c r="D20" s="17"/>
-      <c r="E20" s="17"/>
-      <c r="F20" s="17"/>
-      <c r="G20" s="17"/>
-      <c r="H20" s="17"/>
-      <c r="I20" s="17"/>
-      <c r="J20" s="17"/>
-      <c r="K20" s="17"/>
-      <c r="L20" s="17"/>
-      <c r="M20" s="17"/>
-      <c r="N20" s="17"/>
-      <c r="O20" s="17"/>
-      <c r="P20" s="17"/>
-      <c r="Q20" s="17"/>
-      <c r="R20" s="17"/>
-      <c r="S20" s="17"/>
-      <c r="T20" s="17"/>
-      <c r="U20" s="17"/>
+      <c r="C20" s="13"/>
+      <c r="D20" s="13"/>
+      <c r="E20" s="13"/>
+      <c r="F20" s="13"/>
+      <c r="G20" s="13"/>
+      <c r="H20" s="13"/>
+      <c r="I20" s="13"/>
+      <c r="J20" s="13"/>
+      <c r="K20" s="13"/>
+      <c r="L20" s="13"/>
+      <c r="M20" s="13"/>
+      <c r="N20" s="13"/>
+      <c r="O20" s="13"/>
+      <c r="P20" s="13"/>
+      <c r="Q20" s="13"/>
+      <c r="R20" s="13"/>
+      <c r="S20" s="13"/>
+      <c r="T20" s="13"/>
+      <c r="U20" s="13"/>
     </row>
     <row r="21" s="1" customFormat="true" ht="57.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A21" s="2" t="s">
         <v>316</v>
       </c>
-      <c r="B21" s="17" t="s">
+      <c r="B21" s="13" t="s">
         <v>317</v>
       </c>
-      <c r="C21" s="17"/>
-      <c r="D21" s="17"/>
-      <c r="E21" s="17"/>
-      <c r="F21" s="17"/>
-      <c r="G21" s="17"/>
-      <c r="H21" s="17"/>
-      <c r="I21" s="17"/>
-      <c r="J21" s="17"/>
-      <c r="K21" s="17"/>
-      <c r="L21" s="17"/>
-      <c r="M21" s="17"/>
-      <c r="N21" s="17"/>
-      <c r="O21" s="17"/>
-      <c r="P21" s="17"/>
-      <c r="Q21" s="17"/>
-      <c r="R21" s="17"/>
-      <c r="S21" s="17"/>
-      <c r="T21" s="17"/>
-      <c r="U21" s="17"/>
+      <c r="C21" s="13"/>
+      <c r="D21" s="13"/>
+      <c r="E21" s="13"/>
+      <c r="F21" s="13"/>
+      <c r="G21" s="13"/>
+      <c r="H21" s="13"/>
+      <c r="I21" s="13"/>
+      <c r="J21" s="13"/>
+      <c r="K21" s="13"/>
+      <c r="L21" s="13"/>
+      <c r="M21" s="13"/>
+      <c r="N21" s="13"/>
+      <c r="O21" s="13"/>
+      <c r="P21" s="13"/>
+      <c r="Q21" s="13"/>
+      <c r="R21" s="13"/>
+      <c r="S21" s="13"/>
+      <c r="T21" s="13"/>
+      <c r="U21" s="13"/>
     </row>
     <row r="22" s="1" customFormat="true" ht="57.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A22" s="2" t="s">
         <v>318</v>
       </c>
-      <c r="B22" s="17" t="s">
+      <c r="B22" s="13" t="s">
         <v>319</v>
       </c>
-      <c r="C22" s="17"/>
-      <c r="D22" s="17"/>
-      <c r="E22" s="17"/>
-      <c r="F22" s="17"/>
-      <c r="G22" s="17"/>
-      <c r="H22" s="17"/>
-      <c r="I22" s="17"/>
-      <c r="J22" s="17"/>
-      <c r="K22" s="17"/>
-      <c r="L22" s="17"/>
-      <c r="M22" s="17"/>
-      <c r="N22" s="17"/>
-      <c r="O22" s="17"/>
-      <c r="P22" s="17"/>
-      <c r="Q22" s="17"/>
-      <c r="R22" s="17"/>
-      <c r="S22" s="17"/>
-      <c r="T22" s="17"/>
-      <c r="U22" s="17"/>
+      <c r="C22" s="13"/>
+      <c r="D22" s="13"/>
+      <c r="E22" s="13"/>
+      <c r="F22" s="13"/>
+      <c r="G22" s="13"/>
+      <c r="H22" s="13"/>
+      <c r="I22" s="13"/>
+      <c r="J22" s="13"/>
+      <c r="K22" s="13"/>
+      <c r="L22" s="13"/>
+      <c r="M22" s="13"/>
+      <c r="N22" s="13"/>
+      <c r="O22" s="13"/>
+      <c r="P22" s="13"/>
+      <c r="Q22" s="13"/>
+      <c r="R22" s="13"/>
+      <c r="S22" s="13"/>
+      <c r="T22" s="13"/>
+      <c r="U22" s="13"/>
     </row>
     <row r="23" s="1" customFormat="true" ht="57.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A23" s="2" t="s">
         <v>320</v>
       </c>
-      <c r="B23" s="17" t="s">
+      <c r="B23" s="13" t="s">
         <v>321</v>
       </c>
-      <c r="C23" s="17"/>
-      <c r="D23" s="17"/>
-      <c r="E23" s="17"/>
-      <c r="F23" s="17"/>
-      <c r="G23" s="17"/>
-      <c r="H23" s="17"/>
-      <c r="I23" s="17"/>
-      <c r="J23" s="17"/>
-      <c r="K23" s="17"/>
-      <c r="L23" s="17"/>
-      <c r="M23" s="17"/>
-      <c r="N23" s="17"/>
-      <c r="O23" s="17"/>
-      <c r="P23" s="17"/>
-      <c r="Q23" s="17"/>
-      <c r="R23" s="17"/>
-      <c r="S23" s="17"/>
-      <c r="T23" s="17"/>
-      <c r="U23" s="17"/>
+      <c r="C23" s="13"/>
+      <c r="D23" s="13"/>
+      <c r="E23" s="13"/>
+      <c r="F23" s="13"/>
+      <c r="G23" s="13"/>
+      <c r="H23" s="13"/>
+      <c r="I23" s="13"/>
+      <c r="J23" s="13"/>
+      <c r="K23" s="13"/>
+      <c r="L23" s="13"/>
+      <c r="M23" s="13"/>
+      <c r="N23" s="13"/>
+      <c r="O23" s="13"/>
+      <c r="P23" s="13"/>
+      <c r="Q23" s="13"/>
+      <c r="R23" s="13"/>
+      <c r="S23" s="13"/>
+      <c r="T23" s="13"/>
+      <c r="U23" s="13"/>
     </row>
   </sheetData>
   <mergeCells count="8">
@@ -11506,11 +11490,11 @@
       <c r="A22" s="1" t="s">
         <v>351</v>
       </c>
-      <c r="B22" s="19" t="n">
+      <c r="B22" s="15" t="n">
         <f aca="false">B8*(12.49-1)/(3*12.49)</f>
         <v>0.00358862966714898</v>
       </c>
-      <c r="C22" s="19" t="n">
+      <c r="C22" s="15" t="n">
         <f aca="false">C8*(12.49-1)/(3*12.49)</f>
         <v>0.0177337050363182</v>
       </c>
@@ -11976,128 +11960,126 @@
       </c>
     </row>
     <row r="32" s="1" customFormat="true" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A32" s="11" t="s">
+      <c r="A32" s="1" t="s">
         <v>90</v>
       </c>
-      <c r="B32" s="12" t="n">
+      <c r="B32" s="8" t="n">
         <f aca="false">B16/(B16+B17+B18)</f>
         <v>0.314516129032258</v>
       </c>
-      <c r="C32" s="12" t="n">
+      <c r="C32" s="8" t="n">
         <f aca="false">B17/(B16+B17+B18)</f>
         <v>0.528225806451613</v>
       </c>
-      <c r="D32" s="12" t="n">
+      <c r="D32" s="8" t="n">
         <f aca="false">B18/(B16+B17+B18)</f>
         <v>0.157258064516129</v>
       </c>
-      <c r="E32" s="12" t="n">
+      <c r="E32" s="8" t="n">
         <v>0</v>
       </c>
-      <c r="F32" s="13" t="n">
+      <c r="F32" s="9" t="n">
         <f aca="false">B32*$C$16+C32*$C$17+D32*$C$18+E32*$C$19</f>
         <v>359.258064516129</v>
       </c>
-      <c r="G32" s="13" t="n">
+      <c r="G32" s="9" t="n">
         <f aca="false">B32*$E$16+C32*$E$17+D32*$E$18+E32*$E$19</f>
         <v>47.258064516129</v>
       </c>
     </row>
     <row r="33" s="1" customFormat="true" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A33" s="14" t="s">
+      <c r="A33" s="1" t="s">
         <v>91</v>
       </c>
-      <c r="B33" s="12" t="n">
+      <c r="B33" s="8" t="n">
         <v>0</v>
       </c>
-      <c r="C33" s="12" t="n">
+      <c r="C33" s="8" t="n">
         <v>0</v>
       </c>
-      <c r="D33" s="12" t="n">
+      <c r="D33" s="8" t="n">
         <v>1</v>
       </c>
-      <c r="E33" s="12" t="n">
+      <c r="E33" s="8" t="n">
         <v>0</v>
       </c>
-      <c r="F33" s="13" t="n">
+      <c r="F33" s="9" t="n">
         <f aca="false">B33*$C$16+C33*$C$17+D33*$C$18+E33*$C$19</f>
         <v>319</v>
       </c>
-      <c r="G33" s="13" t="n">
+      <c r="G33" s="9" t="n">
         <f aca="false">B33*$E$16+C33*$E$17+D33*$E$18+E33*$E$19</f>
         <v>0</v>
       </c>
     </row>
-    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A34" s="11" t="s">
+    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A34" s="1" t="s">
         <v>92</v>
       </c>
-      <c r="B34" s="12" t="n">
+      <c r="B34" s="8" t="n">
         <v>1</v>
       </c>
-      <c r="C34" s="12" t="n">
+      <c r="C34" s="8" t="n">
         <v>0</v>
       </c>
-      <c r="D34" s="12" t="n">
+      <c r="D34" s="8" t="n">
         <v>0</v>
       </c>
-      <c r="E34" s="12" t="n">
+      <c r="E34" s="8" t="n">
         <v>0</v>
       </c>
-      <c r="F34" s="13" t="n">
+      <c r="F34" s="9" t="n">
         <f aca="false">B34*$C$16+C34*$C$17+D34*$C$18+E34*$C$19</f>
         <v>447</v>
       </c>
-      <c r="G34" s="13" t="n">
+      <c r="G34" s="9" t="n">
         <f aca="false">B34*$E$16+C34*$E$17+D34*$E$18+E34*$E$19</f>
         <v>73</v>
       </c>
     </row>
-    <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A35" s="11" t="s">
+    <row r="35" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A35" s="1" t="s">
         <v>93</v>
       </c>
-      <c r="B35" s="12" t="n">
+      <c r="B35" s="8" t="n">
         <v>0</v>
       </c>
-      <c r="C35" s="12" t="n">
+      <c r="C35" s="8" t="n">
         <v>1</v>
       </c>
-      <c r="D35" s="12" t="n">
+      <c r="D35" s="8" t="n">
         <v>0</v>
       </c>
-      <c r="E35" s="12" t="n">
+      <c r="E35" s="8" t="n">
         <v>0</v>
       </c>
-      <c r="F35" s="13" t="n">
+      <c r="F35" s="9" t="n">
         <f aca="false">C35*$B$37</f>
         <v>500</v>
       </c>
-      <c r="G35" s="13" t="n">
+      <c r="G35" s="9" t="n">
         <f aca="false">C35*$B$37</f>
         <v>500</v>
       </c>
     </row>
-    <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A37" s="11" t="s">
+    <row r="37" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A37" s="1" t="s">
         <v>94</v>
       </c>
-      <c r="B37" s="13" t="n">
+      <c r="B37" s="9" t="n">
         <v>500</v>
       </c>
-      <c r="D37" s="11" t="s">
+      <c r="D37" s="1" t="s">
         <v>95</v>
       </c>
     </row>
-    <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A39" s="11" t="s">
+    <row r="39" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A39" s="1" t="s">
         <v>96</v>
       </c>
     </row>
-    <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A40" s="11" t="s">
+    <row r="40" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A40" s="1" t="s">
         <v>97</v>
       </c>
     </row>

</xml_diff>